<commit_message>
feat(rq3): blind rater sheets to ground truth/CWE/CVE (FP/FN confound)
With FP/FN in the 4-strata set, showing ground truth/CWE/CVE reveals prediction
(in)correctness and would conflate explanation quality with correctness. Rater
sheets now show only sample_id + source_code + response_text + the 4 Likert cols;
raters judge quality from code + explanation alone. Reuse preserved (30 prior
scores pre-filled, 90 blank). Master frame keeps gt/stratum as the unblinding key.

Note: reused 30 (TP/TN) were rated under the original gt-shown protocol while the
90 new are blinded -> mixed-protocol threat to validity (to be disclosed).
</commit_message>
<xml_diff>
--- a/results/rq3_baseline/fpfn_paired120_rater_HS.xlsx
+++ b/results/rq3_baseline/fpfn_paired120_rater_HS.xlsx
@@ -435,20 +435,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K121"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="80" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,45 +461,30 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ground_truth_label</t>
+          <t>response_text</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>cwe</t>
+          <t>completeness_score</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>cve_desc</t>
+          <t>clarity_score</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>response_text</t>
+          <t>actionability_score</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>completeness_score</t>
+          <t>informativeness_score</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>clarity_score</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>actionability_score</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>informativeness_score</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>rater_notes</t>
         </is>
@@ -528,21 +510,6 @@
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>NULL Pointer Dereference in GitHub repository gpac/gpac prior to 1.1.0.</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 ### Code Analysis
@@ -589,19 +556,19 @@
 **Recommendation**: Verify the structural compatibility of `GF_Box` and `GroupIdToNameBox`, or refactor the code to avoid the cast if possible. Ensure that the memory allocation and deallocation routines are consistent with the actual memory layout being managed.</t>
         </is>
       </c>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="G2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -652,13 +619,6 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Function Purpose:** The function `sctp_make_strreset_req` constructs an SCTP stream reset request chunk. It handles both outgoing (`out`) and incoming (`in`) reset requests based on boolean flags.
@@ -677,11 +637,11 @@
 **Result:** (1) YES: Vulnerability detected.</t>
         </is>
       </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr"/>
       <c r="G3" s="3" t="inlineStr"/>
       <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -752,21 +712,6 @@
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-703']</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>NULL Pointer Dereference in GitHub repository mruby/mruby prior to 3.2.</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step to determine if there's a vulnerability.
 **Code Overview**
@@ -800,11 +745,11 @@
 * If there are specific vulnerability types (e.g., timing attacks, side-channel vulnerabilities) not immediately apparent from the code, a more detailed analysis with those in mind might be necessary.</t>
         </is>
       </c>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
       <c r="G4" s="3" t="inlineStr"/>
       <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -819,21 +764,6 @@
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>fs/seq_file.c in the Linux kernel 3.16 through 5.13.x before 5.13.4 does not properly restrict seq buffer allocations, leading to an integer overflow, an Out-of-bounds Write, and escalation to root by an unprivileged user, aka CID-8cae8cd89f05.</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Explanation:**
@@ -845,11 +775,11 @@
 **Conclusion:** The code is not inherently vulnerable. The function correctly delegates memory allocation to the kernel's memory management system, and the lack of size validation here is not a flaw in isolation. The answer is **NO**.</t>
         </is>
       </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -873,21 +803,6 @@
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>A vulnerability classified as problematic was found in GhostPCL 9.55.0. This vulnerability affects the function chunk_free_object of the file gsmchunk.c. The manipulation with a malicious file leads to a memory corruption. The attack can be initiated remotely but requires user interaction. The exploit has been disclosed to the public as a POC and may be used. It is recommended to apply the patches to fix this issue.</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>### Analysis of the Provided Code
 The function `pcl_status_read` is designed to read data from a buffer managed by the `pcs-&gt;status` structure. It calculates the number of bytes available for reading as the minimum between `max_data` and the difference between `write_pos` and `read_pos`. It then copies that data into the provided `data` buffer and updates the `read_pos` accordingly. If the buffer becomes empty (i.e., `read_pos == write_pos`), it is freed, and both positions are reset to zero.
@@ -922,11 +837,11 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1023,13 +938,6 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Explanation:**
 1. **Initialization Check:** The code checks if the right-hand side tensor (`rhs`) is initialized using `rhs.IsInitialized()`. This prevents use of uninitialized memory, avoiding undefined behavior.
@@ -1045,19 +953,19 @@
 **Answer:** NO</t>
         </is>
       </c>
+      <c r="D7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H7" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -1085,21 +993,6 @@
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>A vulnerability classified as problematic was found in GhostPCL 9.55.0. This vulnerability affects the function chunk_free_object of the file gsmchunk.c. The manipulation with a malicious file leads to a memory corruption. The attack can be initiated remotely but requires user interaction. The exploit has been disclosed to the public as a POC and may be used. It is recommended to apply the patches to fix this issue.</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 **Functionality Overview**
@@ -1141,11 +1034,11 @@
 **Note**: This answer assumes the function is used correctly by callers and does not account for potential issues in the broader context (e.g., multi-threading, initialization of `pcs-&gt;status.buffer`, or the behavior of `gs_free_object`).</t>
         </is>
       </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -1299,13 +1192,6 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 1. **Code Overview**:
 	* The provided code is a method `ParseMCU` within a class `SingleComponentLSScan`.
@@ -1338,11 +1224,11 @@
 - Consider adding overflow/underflow checks for arithmetic operations, especially when dealing with user-controlled data.</t>
         </is>
       </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1428,29 +1314,14 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-119']</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>The bmexec_trans function in kwset.c in grep 2.19 through 2.21 allows local users to cause a denial of service (out-of-bounds heap read and crash) via crafted input when using the -F option.</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
           <t>SKIPPED: timeout</t>
         </is>
       </c>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="3" t="inlineStr"/>
       <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="3" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -1525,21 +1396,6 @@
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-200']</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>The openssl_encrypt function in ext/openssl/openssl.c in PHP 5.3.9 through 5.3.13 does not initialize a certain variable, which allows remote attackers to obtain sensitive information from process memory by providing zero bytes of input data.</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided PHP extension code for the `openssl_encrypt` function step by step to determine if there's a vulnerability.
 ### Step 1: Parameter Parsing
@@ -1570,11 +1426,11 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -1866,13 +1722,6 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 1. **Code Overview**:
 	* The provided code is a C function `EC_GROUP_new_from_ecparameters` from OpenSSL, which creates an `EC_GROUP` object from given elliptic curve parameters.
@@ -1899,11 +1748,11 @@
 **Note**: This analysis is based on the code snippet provided and assumes that the underlying OpenSSL library functions are secure and that the code is used in a secure context. A comprehensive security audit would require analyzing the entire codebase and its usage context.</t>
         </is>
       </c>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
       <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1934,13 +1783,6 @@
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 **Code Overview**
@@ -1972,11 +1814,11 @@
 - Ensure `buf` is NULL-checked and that its size is at least `len` bytes before performing the `memcpy`. This might involve adding a parameter for `buf` size or using a safer copy function if available.</t>
         </is>
       </c>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -2288,13 +2130,6 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
           <t>YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Buffer Overflow in Order List Processing:**
@@ -2309,11 +2144,11 @@
 **Conclusion:** The code contains a buffer overflow vulnerability in the handling of the order list, making it vulnerable to exploitation by a maliciously crafted S3M file.</t>
         </is>
       </c>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -2662,13 +2497,6 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
           <t>NO: No vulnerability detected.
 The provided code is part of Vim's command parsing logic, specifically handling command modifiers and Visual mode ranges. After a detailed analysis:
 1. **Buffer Handling**: The code modifies the command string in-place (e.g., moving the Visual range `'&lt;,'&gt;`). While this involves `mch_memmove` operations, Vim's internal buffer management typically ensures sufficient space, and the code checks for valid pointers and lengths.
@@ -2681,19 +2509,19 @@
 **Answer:** NO</t>
         </is>
       </c>
+      <c r="D15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G15" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I15" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J15" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -2768,21 +2596,6 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-362']</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>World-writable permissions on the /tmp/tmate/sessions directory in tmate-ssh-server 2.3.0 allow a local attacker to compromise the integrity of session handling, or obtain the read-write session ID from a read-only session symlink in this directory.</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
           <t>YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Uninitialized Global Pointer (`tmate_settings`):**  
@@ -2797,11 +2610,11 @@
 The lack of initialization for the global pointer `tmate_settings` leads to a NULL pointer dereference when any command-line option is processed. This is a clear vulnerability that can be exploited to crash the program, making the answer **YES: Vulnerability detected**.</t>
         </is>
       </c>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
       <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
-      <c r="J16" s="3" t="inlineStr"/>
-      <c r="K16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -3890,13 +3703,6 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
           <t>The provided code contains a potential **stack buffer overflow vulnerability** due to insufficient bounds checking on the `depth` variable when accessing the `stack` array.
 ### Key Analysis:
 1. **Stack Array Declaration**:
@@ -3924,11 +3730,11 @@
 **Answer:** YES</t>
         </is>
       </c>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="inlineStr"/>
       <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr"/>
-      <c r="J17" s="3" t="inlineStr"/>
-      <c r="K17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -3990,13 +3796,6 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
           <t>YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Insufficient Length Check in Initial Validation:**
@@ -4013,11 +3812,11 @@
 The code contains a vulnerability due to insufficient validation of the `skb` buffer length before accessing its data. This can lead to out-of-bounds memory accesses, making the code vulnerable to exploitation.</t>
         </is>
       </c>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
       <c r="G18" s="3" t="inlineStr"/>
       <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr"/>
-      <c r="K18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -4103,21 +3902,6 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-119']</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>The bmexec_trans function in kwset.c in grep 2.19 through 2.21 allows local users to cause a denial of service (out-of-bounds heap read and crash) via crafted input when using the -F option.</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
 The function `bmexec_trans` appears to be part of a string searching algorithm, likely an optimized variant of the Boyer-Moore algorithm, given the use of delta (difference) tables and heuristics for skipping characters. It searches for a pattern (defined by `kwset`) within a text buffer (`text` of size `size`).
@@ -4141,11 +3925,11 @@
 **Caveat**: This analysis is based on the provided code snippet and assumes the surrounding code and environment (e.g., how `kwset` is initialized, the implementation of `memchr_kwset`, and the `bm_delta2_search` function) do not introduce vulnerabilities. A full codebase review would be necessary for absolute certainty.</t>
         </is>
       </c>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
       <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="3" t="inlineStr"/>
-      <c r="K19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -4246,13 +4030,6 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 **Code Overview**
 ----------------
@@ -4283,11 +4060,11 @@
 - Review the system's configuration and the process's privileges to ensure they align with the principle of least privilege, especially regarding file operations.</t>
         </is>
       </c>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
       <c r="G20" s="3" t="inlineStr"/>
       <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="3" t="inlineStr"/>
-      <c r="K20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -4316,13 +4093,6 @@
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
@@ -4344,11 +4114,11 @@
 Answer: (1) YES: Vulnerability detected.</t>
         </is>
       </c>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
       <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr"/>
-      <c r="J21" s="3" t="inlineStr"/>
-      <c r="K21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -4370,21 +4140,6 @@
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>NULL Pointer Dereference in GitHub repository gpac/gpac prior to 1.1.0.</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
@@ -4398,19 +4153,19 @@
 **Result:** YES (Vulnerability detected).</t>
         </is>
       </c>
+      <c r="D22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="G22" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I22" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J22" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -4700,13 +4455,6 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
           <t>**Security Analysis of Provided Code**
 ### Step-by-Step Review
 1. **Input Validation**:
@@ -4737,11 +4485,11 @@
 ```</t>
         </is>
       </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
       <c r="G23" s="3" t="inlineStr"/>
       <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr"/>
-      <c r="K23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -4828,21 +4576,6 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-703']</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>A packet of death scenario is possible in mvfst via a specially crafted message during a QUIC session, which causes a crash via a failed assertion. Per QUIC specification, this particular message should be treated as a connection error. This issue affects mvfst versions prior to commit a67083ff4b8dcbb7ee2839da6338032030d712b0 and proxygen versions prior to v2021.03.15.00.</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Explanation:**
 1. **Null Pointer Checks:** The code checks each cipher (e.g., `zeroRttReadCipher`, `oneRttWriteCipher`) for null before using it. This prevents null pointer dereferences.
@@ -4855,11 +4588,11 @@
 No memory safety issues, logic errors, or security flaws (e.g., buffer overflows, use-after-free, or improper key handling) are present in the code. The code follows best practices for resource management and state transitions in a QUIC implementation.</t>
         </is>
       </c>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
       <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr"/>
-      <c r="J24" s="3" t="inlineStr"/>
-      <c r="K24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -4934,21 +4667,6 @@
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-200']</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>The openssl_encrypt function in ext/openssl/openssl.c in PHP 5.3.9 through 5.3.13 does not initialize a certain variable, which allows remote attackers to obtain sensitive information from process memory by providing zero bytes of input data.</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>### Analysis of the Provided PHP Code
 The code in question is an implementation of the `openssl_encrypt` function in PHP, which performs encryption using OpenSSL. The goal is to determine whether this code contains any vulnerabilities that could lead to security issues such as memory corruption, buffer overflows, or incorrect encryption behavior.
@@ -4990,11 +4708,11 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
       <c r="G25" s="3" t="inlineStr"/>
       <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr"/>
-      <c r="J25" s="3" t="inlineStr"/>
-      <c r="K25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -5018,21 +4736,6 @@
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Tensorflow is an Open Source Machine Learning Framework. Under certain scenarios, Grappler component of TensorFlow can trigger a null pointer dereference. There are 2 places where this can occur, for the same malicious alteration of a `SavedModel` file (fixing the first one would trigger the same dereference in the second place). First, during constant folding, the `GraphDef` might not have the required nodes for the binary operation. If a node is missing, the correposning `mul_*child` would be null, and the dereference in the subsequent line would be incorrect. We have a similar issue during `IsIdentityConsumingSwitch`. The fix will be included in TensorFlow 2.8.0. We will also cherrypick this commit on TensorFlow 2.7.1, TensorFlow 2.6.3, and TensorFlow 2.5.3, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step to determine if there's a vulnerability.
 **Code Snippet Analysis**
@@ -5088,19 +4791,19 @@
 ```</t>
         </is>
       </c>
+      <c r="D26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="G26" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H26" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="I26" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J26" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -5152,21 +4855,6 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-369']</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>In Deark before v1.5.8, a specially crafted input file can cause a division by zero in (src/fmtutil.c) because of the value of pixelsize.</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
 The function `fmtutil_macbitmap_read_pixmap_only_fields` reads specific fields from a PixMap header in a file (or buffer) at a given position (`pos`). It extracts various metadata related to a MacBitmap image, such as version, packing type, pixel data length, DPI, pixel format, and more, storing these in a `struct fmtutil_macbitmap_info` object (`bi`).
@@ -5196,19 +4884,19 @@
 - Consider adding bounds checks and sanitization for all data originating from untrusted sources.</t>
         </is>
       </c>
+      <c r="D27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="I27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J27" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -5243,13 +4931,6 @@
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>### Step-by-Step Analysis
 The function `dynamicGetbuf` is designed to read data from a dynamically allocated buffer managed by a `dynamicPtr` structure. It takes three parameters: a context pointer `ctx`, a buffer `buf` to store the result, and the number of bytes `len` to read. The function returns the number of bytes read or `EOF` if no more data is available.
@@ -5286,11 +4967,11 @@
 **(1) YES: Vulnerability detected.**</t>
         </is>
       </c>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
       <c r="G28" s="3" t="inlineStr"/>
       <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -5387,13 +5068,6 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
           <t>YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Unvalidated Input Parameters:**
@@ -5409,11 +5083,11 @@
 **Answer:** YES</t>
         </is>
       </c>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
       <c r="G29" s="3" t="inlineStr"/>
       <c r="H29" s="3" t="inlineStr"/>
-      <c r="I29" s="3" t="inlineStr"/>
-      <c r="J29" s="3" t="inlineStr"/>
-      <c r="K29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -5440,21 +5114,6 @@
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>Buffer overflow in the send_control_msg function in hw/char/virtio-serial-bus.c in QEMU before 2.4.0 allows guest users to cause a denial of service (QEMU process crash) via a crafted virtio control message.</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
@@ -5472,11 +5131,11 @@
 **Answer:** (1) YES: Vulnerability detected.</t>
         </is>
       </c>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
       <c r="G30" s="3" t="inlineStr"/>
       <c r="H30" s="3" t="inlineStr"/>
-      <c r="I30" s="3" t="inlineStr"/>
-      <c r="J30" s="3" t="inlineStr"/>
-      <c r="K30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -5570,13 +5229,6 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Buffer Overflow in `szLineConv` (Unicode Type &lt;=1):**
@@ -5590,11 +5242,11 @@
 **Conclusion:** The code contains buffer overflow vulnerabilities in both branches of the Unicode type handling due to insufficient bounds checking on the fixed-size `szLineConv` buffer. This allows an attacker to corrupt memory, potentially leading to crashes or arbitrary code execution.</t>
         </is>
       </c>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
       <c r="G31" s="3" t="inlineStr"/>
       <c r="H31" s="3" t="inlineStr"/>
-      <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="inlineStr"/>
-      <c r="K31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -5715,21 +5367,6 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-189']</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>Multiple integer overflows in the read_bitmap_file_data function in io-xbm.c in gdk-pixbuf before 2.26.1 allow remote attackers to cause a denial of service (application crash) via a negative (1) height or (2) width in an XBM file, which triggers a heap-based buffer overflow.</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
 The `read_bitmap_file_data` function reads a bitmap file, extracts its width, height, data, and optional hotspots (x_hot, y_hot). It supports both old and new formats of bitmap files.
@@ -5758,11 +5395,11 @@
 	* Although not shown, ensure the `next_int` function is secure and doesn’t introduce vulnerabilities (e.g., buffer overreads).</t>
         </is>
       </c>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr"/>
       <c r="G32" s="3" t="inlineStr"/>
       <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr"/>
-      <c r="J32" s="3" t="inlineStr"/>
-      <c r="K32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -6173,23 +5810,16 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
           <t>After a thorough analysis of the provided code, no critical vulnerabilities such as buffer overflows, memory leaks, or exploitable VULNERABILITIES were identified. The code demonstrates robust error handling, proper memory management (with cleanup in error paths), and validation of critical parameters (e.g., tile dimensions, resolution levels, and layer rates). While there are minor concerns like the use of `atoi` without error checking and potential integer overflows in edge cases (e.g., large image components or malformed input), these do not constitute exploitable vulnerabilities under typical usage scenarios. The code adheres to safe practices for memory allocation and input validation, ensuring no direct security risks.
 **Answer:**  
 NO</t>
         </is>
       </c>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
       <c r="G33" s="3" t="inlineStr"/>
       <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr"/>
-      <c r="J33" s="3" t="inlineStr"/>
-      <c r="K33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -6288,13 +5918,6 @@
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
@@ -6319,19 +5942,19 @@
 **Result: (2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D34" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G34" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H34" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I34" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J34" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -6436,13 +6059,6 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
           <t>### Analysis of the Provided Code
 The function `set_fflags_platform` is designed to set file flags (e.g., immutable, append-only) on a file or directory using Linux-specific `ioctl` operations. It handles both the case where a file descriptor is provided and where it must open the file itself. The code includes several safety measures and error-handling mechanisms.
 ---
@@ -6484,11 +6100,11 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr"/>
       <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr"/>
-      <c r="J35" s="3" t="inlineStr"/>
-      <c r="K35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -6535,13 +6151,6 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr"/>
-      <c r="E36" s="3" t="inlineStr"/>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Buffer Overflow in `dst` Buffer:**
@@ -6555,11 +6164,11 @@
 (1) YES: Vulnerability detected.</t>
         </is>
       </c>
+      <c r="D36" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr"/>
       <c r="G36" s="3" t="inlineStr"/>
       <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr"/>
-      <c r="J36" s="3" t="inlineStr"/>
-      <c r="K36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -6604,13 +6213,6 @@
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
@@ -6635,19 +6237,19 @@
 **Note**: This analysis might change with additional context or the implementation details of `__get_clean_virt` and `memslot_validate_virt`. For a comprehensive security audit, reviewing the entire codebase and understanding the project's specific requirements and constraints is essential.</t>
         </is>
       </c>
+      <c r="D37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="G37" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H37" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I37" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J37" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -6697,13 +6299,6 @@
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr"/>
-      <c r="E38" s="3" t="inlineStr"/>
-      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Functionality Overview**
@@ -6747,11 +6342,11 @@
 **Result: (1) YES: Vulnerability detected.**</t>
         </is>
       </c>
+      <c r="D38" s="3" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr"/>
+      <c r="F38" s="3" t="inlineStr"/>
       <c r="G38" s="3" t="inlineStr"/>
       <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="3" t="inlineStr"/>
-      <c r="J38" s="3" t="inlineStr"/>
-      <c r="K38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -6922,13 +6517,6 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr"/>
-      <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Analysis:**
 1. **Input Validation:**
@@ -6949,19 +6537,19 @@
 Answer: (2) NO</t>
         </is>
       </c>
+      <c r="D39" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G39" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H39" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I39" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J39" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -7251,13 +6839,6 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr"/>
-      <c r="E40" s="3" t="inlineStr"/>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
           <t>YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Buffer Overflow in `sprintf` Usage:**
@@ -7274,11 +6855,11 @@
 **Conclusion:** The use of `sprintf` with a fixed-size buffer and untrusted input data introduces a buffer overflow vulnerability.</t>
         </is>
       </c>
+      <c r="D40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr"/>
+      <c r="F40" s="3" t="inlineStr"/>
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr"/>
-      <c r="I40" s="3" t="inlineStr"/>
-      <c r="J40" s="3" t="inlineStr"/>
-      <c r="K40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -7323,13 +6904,6 @@
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Analysis:**
@@ -7352,19 +6926,19 @@
 (2) NO: No vulnerability.</t>
         </is>
       </c>
+      <c r="D41" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="G41" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H41" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I41" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J41" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -7474,13 +7048,6 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr"/>
-      <c r="E42" s="3" t="inlineStr"/>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
 ----------------
@@ -7513,11 +7080,11 @@
 - Enhance error messages for better debugging support.</t>
         </is>
       </c>
+      <c r="D42" s="3" t="inlineStr"/>
+      <c r="E42" s="3" t="inlineStr"/>
+      <c r="F42" s="3" t="inlineStr"/>
       <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr"/>
-      <c r="I42" s="3" t="inlineStr"/>
-      <c r="J42" s="3" t="inlineStr"/>
-      <c r="K42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -7534,13 +7101,6 @@
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr"/>
-      <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step to determine if it contains a vulnerability.
 ### Code Snippet:
@@ -7575,11 +7135,11 @@
 **Note**: For a comprehensive security analysis, the definitions of `ADD_ALL_TESTS`, `OSSL_NELEM`, `ADD_TEST`, and `name_fns` should be reviewed.</t>
         </is>
       </c>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="3" t="inlineStr"/>
+      <c r="F43" s="3" t="inlineStr"/>
       <c r="G43" s="3" t="inlineStr"/>
       <c r="H43" s="3" t="inlineStr"/>
-      <c r="I43" s="3" t="inlineStr"/>
-      <c r="J43" s="3" t="inlineStr"/>
-      <c r="K43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -7652,13 +7212,6 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr"/>
-      <c r="E44" s="3" t="inlineStr"/>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Input Validation in Release Builds:**
@@ -7673,11 +7226,11 @@
 **Conclusion:** The code is vulnerable due to insufficient bounds checking in release builds, which can lead to exceptions and crashes when processing malformed input.</t>
         </is>
       </c>
+      <c r="D44" s="3" t="inlineStr"/>
+      <c r="E44" s="3" t="inlineStr"/>
+      <c r="F44" s="3" t="inlineStr"/>
       <c r="G44" s="3" t="inlineStr"/>
       <c r="H44" s="3" t="inlineStr"/>
-      <c r="I44" s="3" t="inlineStr"/>
-      <c r="J44" s="3" t="inlineStr"/>
-      <c r="K44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
@@ -7773,21 +7326,6 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-119']</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>Stack consumption vulnerability in GD in PHP before 5.6.12 allows remote attackers to cause a denial of service via a crafted imagefilltoborder call.</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Recursive Function Calls:**  
@@ -7806,11 +7344,11 @@
 (1) YES: Vulnerability detected.</t>
         </is>
       </c>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr"/>
       <c r="G45" s="3" t="inlineStr"/>
       <c r="H45" s="3" t="inlineStr"/>
-      <c r="I45" s="3" t="inlineStr"/>
-      <c r="J45" s="3" t="inlineStr"/>
-      <c r="K45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -8899,13 +8437,6 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr"/>
-      <c r="E46" s="3" t="inlineStr"/>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 Given the provided code snippet, which appears to be a part of a spell checking or suggestion system (likely from Vim, given the style and some function names), we will analyze it for potential vulnerabilities.
 ### 1. **Code Overview**
@@ -8934,11 +8465,11 @@
 - Ensure all string operations use length-limited functions (e.g., `strncpy` instead of `strcpy`).</t>
         </is>
       </c>
+      <c r="D46" s="3" t="inlineStr"/>
+      <c r="E46" s="3" t="inlineStr"/>
+      <c r="F46" s="3" t="inlineStr"/>
       <c r="G46" s="3" t="inlineStr"/>
       <c r="H46" s="3" t="inlineStr"/>
-      <c r="I46" s="3" t="inlineStr"/>
-      <c r="J46" s="3" t="inlineStr"/>
-      <c r="K46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -9136,13 +8667,6 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr"/>
-      <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 ### 1. **Code Overview**
 The provided code is a function named `change_indent`, which appears to be part of a text editor (likely Vim, given the naming conventions and functions used). The function adjusts the indentation of a line in the editor based on various parameters.
@@ -9166,11 +8690,11 @@
 **Note:** This analysis is based on the provided code snippet and assumes the surrounding code and environment do not mitigate the identified concerns. A full audit of the entire codebase would be necessary for a comprehensive vulnerability assessment.</t>
         </is>
       </c>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr"/>
       <c r="G47" s="3" t="inlineStr"/>
       <c r="H47" s="3" t="inlineStr"/>
-      <c r="I47" s="3" t="inlineStr"/>
-      <c r="J47" s="3" t="inlineStr"/>
-      <c r="K47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -9265,21 +8789,6 @@
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-119']</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>Stack consumption vulnerability in GD in PHP before 5.6.12 allows remote attackers to cause a denial of service via a crafted imagefilltoborder call.</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step to determine if it contains a vulnerability.
 **Code Overview**
@@ -9306,11 +8815,11 @@
 2. **Implement Iterative Approach for Deep Recursions**: To prevent potential stack overflows, consider converting the recursive logic for filling above and below into an iterative approach using a stack or queue data structure.</t>
         </is>
       </c>
+      <c r="D48" s="3" t="inlineStr"/>
+      <c r="E48" s="3" t="inlineStr"/>
+      <c r="F48" s="3" t="inlineStr"/>
       <c r="G48" s="3" t="inlineStr"/>
       <c r="H48" s="3" t="inlineStr"/>
-      <c r="I48" s="3" t="inlineStr"/>
-      <c r="J48" s="3" t="inlineStr"/>
-      <c r="K48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -9409,13 +8918,6 @@
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr"/>
-      <c r="E49" s="2" t="inlineStr"/>
-      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Explanation:**
@@ -9442,19 +8944,19 @@
 (2) NO: No vulnerability.</t>
         </is>
       </c>
+      <c r="D49" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G49" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H49" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I49" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J49" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K49" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -9544,21 +9046,6 @@
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-703']</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>A packet of death scenario is possible in mvfst via a specially crafted message during a QUIC session, which causes a crash via a failed assertion. Per QUIC specification, this particular message should be treated as a connection error. This issue affects mvfst versions prior to commit a67083ff4b8dcbb7ee2839da6338032030d712b0 and proxygen versions prior to v2021.03.15.00.</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step from a **static program analysis** and **security** perspective.
 ---
@@ -9608,11 +9095,11 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D50" s="3" t="inlineStr"/>
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="3" t="inlineStr"/>
       <c r="G50" s="3" t="inlineStr"/>
       <c r="H50" s="3" t="inlineStr"/>
-      <c r="I50" s="3" t="inlineStr"/>
-      <c r="J50" s="3" t="inlineStr"/>
-      <c r="K50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -9662,21 +9149,6 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>mruby is vulnerable to NULL Pointer Dereference</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Explanation:**
 1. **Function Purpose:** The function `mrb_ary_shift_m` implements the array shift operation in the Mr. Ruby (mrb) interpreter, removing the first `n` elements from the array and returning them as a new array.
@@ -9698,11 +9170,11 @@
 (2) NO: No vulnerability.</t>
         </is>
       </c>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="3" t="inlineStr"/>
+      <c r="F51" s="3" t="inlineStr"/>
       <c r="G51" s="3" t="inlineStr"/>
       <c r="H51" s="3" t="inlineStr"/>
-      <c r="I51" s="3" t="inlineStr"/>
-      <c r="J51" s="3" t="inlineStr"/>
-      <c r="K51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -9740,21 +9212,6 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-416']</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>TensorFlow is an end-to-end open source platform for machine learning. In affected versions the implementation for `tf.raw_ops.BoostedTreesCreateEnsemble` can result in a use after free error if an attacker supplies specially crafted arguments. The [implementation](https://github.com/tensorflow/tensorflow/blob/f24faa153ad31a4b51578f8181d3aaab77a1ddeb/tensorflow/core/kernels/boosted_trees/resource_ops.cc#L55) uses a reference counted resource and decrements the refcount if the initialization fails, as it should. However, when the code was written, the resource was represented as a naked pointer but later refactoring has changed it to be a smart pointer. Thus, when the pointer leaves the scope, a subsequent `free`-ing of the resource occurs, but this fails to take into account that the refcount has already reached 0, thus the resource has been already freed. During this double-free process, members of the resource object are accessed for cleanup but they are invalid as the entire resource has been freed. We have patched the issue in GitHub commit 5ecec9c6fbdbc6be03295685190a45e7eee726ab. The fix will be included in TensorFlow 2.6.0. We will also cherrypick this commit on TensorFlow 2.5.1, TensorFlow 2.4.3, and TensorFlow 2.3.4, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Resource Management with `unique_ptr`:**  
@@ -9771,11 +9228,11 @@
 The code contains a double-free vulnerability due to improper handling of reference-counted objects with `unique_ptr`. This is a critical memory safety issue that could lead to crashes or arbitrary code execution.</t>
         </is>
       </c>
+      <c r="D52" s="3" t="inlineStr"/>
+      <c r="E52" s="3" t="inlineStr"/>
+      <c r="F52" s="3" t="inlineStr"/>
       <c r="G52" s="3" t="inlineStr"/>
       <c r="H52" s="3" t="inlineStr"/>
-      <c r="I52" s="3" t="inlineStr"/>
-      <c r="J52" s="3" t="inlineStr"/>
-      <c r="K52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -9799,21 +9256,6 @@
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Tensorflow is an Open Source Machine Learning Framework. Under certain scenarios, Grappler component of TensorFlow can trigger a null pointer dereference. There are 2 places where this can occur, for the same malicious alteration of a `SavedModel` file (fixing the first one would trigger the same dereference in the second place). First, during constant folding, the `GraphDef` might not have the required nodes for the binary operation. If a node is missing, the correposning `mul_*child` would be null, and the dereference in the subsequent line would be incorrect. We have a similar issue during `IsIdentityConsumingSwitch`. The fix will be included in TensorFlow 2.8.0. We will also cherrypick this commit on TensorFlow 2.7.1, TensorFlow 2.6.3, and TensorFlow 2.5.3, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
@@ -9833,19 +9275,19 @@
 Answer: (1) YES: Vulnerability detected.</t>
         </is>
       </c>
+      <c r="D53" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="G53" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H53" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I53" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J53" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K53" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -9967,13 +9409,6 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr"/>
-      <c r="E54" s="3" t="inlineStr"/>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
           <t>After a thorough analysis of the provided code, the following observations and conclusions are made:
 1. **Buffer Handling**: The code uses a fixed-size buffer (`buffer`) to store directory entries and their names. The buffer size is calculated as `sizeof(squashfs_dir_entry_2) + SQUASHFS_NAME_LEN + 1`, which accounts for the maximum allowed name length (`SQUASHFS_NAME_LEN`) plus a null terminator. The code checks that `dire-&gt;size &lt; SQUASHFS_NAME_LEN` before copying the name, ensuring that the name fits within the allocated buffer. Additionally, the code explicitly null-terminates the name, preventing potential buffer overflows during string operations.
 2. **Input Validation**: The code validates critical values such as `dir_count` (ensuring it does not exceed `SQUASHFS_DIR_COUNT`) and `dire-&gt;size` (ensuring it is less than `SQUASHFS_NAME_LEN`). These checks prevent excessive memory allocation and handle malformed filesystem data gracefully.
@@ -9986,11 +9421,11 @@
 (2) NO: No vulnerability.</t>
         </is>
       </c>
+      <c r="D54" s="3" t="inlineStr"/>
+      <c r="E54" s="3" t="inlineStr"/>
+      <c r="F54" s="3" t="inlineStr"/>
       <c r="G54" s="3" t="inlineStr"/>
       <c r="H54" s="3" t="inlineStr"/>
-      <c r="I54" s="3" t="inlineStr"/>
-      <c r="J54" s="3" t="inlineStr"/>
-      <c r="K54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
@@ -10107,21 +9542,6 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-120']</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>A buffer overflow vulnerability in jetp3852_print_page() in devices/gdev3852.c of Artifex Software GhostScript v9.50 allows a remote attacker to escalate privileges via a crafted PDF file. This is fixed in v9.51.</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
           <t>The provided code for the `jetp3852_print_page` function appears to be a printer driver implementation, likely part of the Ghostscript project. After a detailed analysis of the code, the following observations and conclusions were made:
 ### Key Observations:
 1. **Buffer Size Validation**:
@@ -10143,11 +9563,11 @@
 No vulnerability was detected in the provided code.</t>
         </is>
       </c>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr"/>
+      <c r="F55" s="3" t="inlineStr"/>
       <c r="G55" s="3" t="inlineStr"/>
       <c r="H55" s="3" t="inlineStr"/>
-      <c r="I55" s="3" t="inlineStr"/>
-      <c r="J55" s="3" t="inlineStr"/>
-      <c r="K55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n">
@@ -10246,21 +9666,6 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-125']</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>An out-of-bounds read flaw was found in the Linux kernel’s io_uring module in the way a user triggers the io_read() function with some special parameters. This flaw allows a local user to read some memory out of bounds.</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
           <t>YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Memory Allocation Context:**
@@ -10274,11 +9679,11 @@
 **Conclusion:** The code incorrectly frees stack-allocated memory in error and cleanup paths, leading to a vulnerability.</t>
         </is>
       </c>
+      <c r="D56" s="3" t="inlineStr"/>
+      <c r="E56" s="3" t="inlineStr"/>
+      <c r="F56" s="3" t="inlineStr"/>
       <c r="G56" s="3" t="inlineStr"/>
       <c r="H56" s="3" t="inlineStr"/>
-      <c r="I56" s="3" t="inlineStr"/>
-      <c r="J56" s="3" t="inlineStr"/>
-      <c r="K56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -10421,13 +9826,6 @@
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr"/>
-      <c r="E57" s="3" t="inlineStr"/>
-      <c r="F57" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
@@ -10456,11 +9854,11 @@
 **Answer: NO**</t>
         </is>
       </c>
+      <c r="D57" s="3" t="inlineStr"/>
+      <c r="E57" s="3" t="inlineStr"/>
+      <c r="F57" s="3" t="inlineStr"/>
       <c r="G57" s="3" t="inlineStr"/>
       <c r="H57" s="3" t="inlineStr"/>
-      <c r="I57" s="3" t="inlineStr"/>
-      <c r="J57" s="3" t="inlineStr"/>
-      <c r="K57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -10620,21 +10018,6 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>TensorFlow is an open source platform for machine learning. Prior to versions 2.9.0, 2.8.1, 2.7.2, and 2.6.4, the implementation of `tf.raw_ops.EditDistance` has incomplete validation. Users can pass negative values to cause a segmentation fault based denial of service. In multiple places throughout the code, one may compute an index for a write operation. However, the existing validation only checks against the upper bound of the array. Hence, it is possible to write before the array by massaging the input to generate negative values for `loc`. Versions 2.9.0, 2.8.1, 2.7.2, and 2.6.4 contain a patch for this issue.</t>
-        </is>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Analysis:**
 1. **Input Validation:**  
@@ -10659,11 +10042,11 @@
 The code rigorously validates inputs, ensures memory safety through bounds checks, and uses TensorFlow's robust error handling mechanisms. No vulnerabilities (e.g., buffer overflows, use-after-free, or uninitialized memory access) are present. The answer is **NO**.</t>
         </is>
       </c>
+      <c r="D58" s="3" t="inlineStr"/>
+      <c r="E58" s="3" t="inlineStr"/>
+      <c r="F58" s="3" t="inlineStr"/>
       <c r="G58" s="3" t="inlineStr"/>
       <c r="H58" s="3" t="inlineStr"/>
-      <c r="I58" s="3" t="inlineStr"/>
-      <c r="J58" s="3" t="inlineStr"/>
-      <c r="K58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -10877,13 +10260,6 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr"/>
-      <c r="E59" s="2" t="inlineStr"/>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
           <t>NO: No vulnerability.
 The code for `pjmedia_rtcp_xr_rx_rtcp_xr` demonstrates careful handling of input validation and buffer boundaries. Key points include:
 1. **RTCP Packet Length Validation**: The function checks that the RTCP packet length (`pkt_len`) is within the provided buffer size (`size`) using `(pkt_len + 1) &gt; (size / 4)`, ensuring the packet does not exceed the allocated memory.
@@ -10902,19 +10278,19 @@
 **Result**: NO</t>
         </is>
       </c>
+      <c r="D59" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G59" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H59" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I59" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J59" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K59" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -11019,21 +10395,6 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-369']</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>TensorFlow is an end-to-end open source platform for machine learning. In affected versions an attacker can craft a TFLite model that would trigger a null pointer dereference, which would result in a crash and denial of service. The [implementation](https://github.com/tensorflow/tensorflow/blob/149562d49faa709ea80df1d99fc41d005b81082a/tensorflow/lite/kernels/internal/optimized/optimized_ops.h#L268-L285) unconditionally dereferences a pointer. We have patched the issue in GitHub commit 15691e456c7dc9bd6be203b09765b063bf4a380c. The fix will be included in TensorFlow 2.6.0. We will also cherrypick this commit on TensorFlow 2.5.1, TensorFlow 2.4.3, and TensorFlow 2.3.4, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Lack of Input Validation:** The function uses `params.broadcast_shape` (dimensions y0-y4) to control loop iterations and pointer arithmetic. However, it does not validate these dimensions against the actual input shapes (`unswitched_input1_shape`, `unswitched_input2_shape`) provided as parameters. This allows for potential out-of-bounds memory access if the broadcast shape is miscalculated or maliciously crafted.
@@ -11044,19 +10405,19 @@
 Answer: (1) YES</t>
         </is>
       </c>
+      <c r="D60" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G60" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H60" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I60" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J60" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K60" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -11173,21 +10534,6 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-369']</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>Tensorflow is an Open Source Machine Learning Framework. The implementation of `FractionalMaxPool` can be made to crash a TensorFlow process via a division by 0. The fix will be included in TensorFlow 2.8.0. We will also cherrypick this commit on TensorFlow 2.7.1, TensorFlow 2.6.3, and TensorFlow 2.5.3, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 **Code Overview**
 The code is a method `Compute` of a class, likely part of a deep learning framework (given the use of `OpKernelContext` and `Tensor`), implementing a custom pooling operation (similar to max pooling) with optional overlapping. It processes a 4D input tensor and produces 3 output tensors: the pooled feature map and two sequences describing the pooling regions for height and width.
@@ -11216,11 +10562,11 @@
 **Result:** **NO** (No vulnerability detected)</t>
         </is>
       </c>
+      <c r="D61" s="3" t="inlineStr"/>
+      <c r="E61" s="3" t="inlineStr"/>
+      <c r="F61" s="3" t="inlineStr"/>
       <c r="G61" s="3" t="inlineStr"/>
       <c r="H61" s="3" t="inlineStr"/>
-      <c r="I61" s="3" t="inlineStr"/>
-      <c r="J61" s="3" t="inlineStr"/>
-      <c r="K61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n">
@@ -11290,13 +10636,6 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr"/>
-      <c r="E62" s="3" t="inlineStr"/>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Input and Segment ID Validation:**
@@ -11312,11 +10651,11 @@
 Answer: (1) YES</t>
         </is>
       </c>
+      <c r="D62" s="3" t="inlineStr"/>
+      <c r="E62" s="3" t="inlineStr"/>
+      <c r="F62" s="3" t="inlineStr"/>
       <c r="G62" s="3" t="inlineStr"/>
       <c r="H62" s="3" t="inlineStr"/>
-      <c r="I62" s="3" t="inlineStr"/>
-      <c r="J62" s="3" t="inlineStr"/>
-      <c r="K62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -11385,13 +10724,6 @@
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr"/>
-      <c r="E63" s="3" t="inlineStr"/>
-      <c r="F63" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
@@ -11440,11 +10772,11 @@
 This check ensures that `output_index` is within the valid range of `output_flat`, preventing potential buffer overflows.</t>
         </is>
       </c>
+      <c r="D63" s="3" t="inlineStr"/>
+      <c r="E63" s="3" t="inlineStr"/>
+      <c r="F63" s="3" t="inlineStr"/>
       <c r="G63" s="3" t="inlineStr"/>
       <c r="H63" s="3" t="inlineStr"/>
-      <c r="I63" s="3" t="inlineStr"/>
-      <c r="J63" s="3" t="inlineStr"/>
-      <c r="K63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -11470,13 +10802,6 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr"/>
-      <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Explanation:**
 1. **Null Pointer Check:** The code checks `if (prog)` before accessing `prog-&gt;type`, preventing null pointer dereference.
@@ -11488,19 +10813,19 @@
 **Conclusion:** The provided code does not exhibit direct vulnerabilities like buffer overflows, null pointer dereferences, or unsafe memory access. Potential issues (e.g., global state modification, external function safety) are either design choices or require additional context not provided. Thus, no vulnerability is detected in the given code.</t>
         </is>
       </c>
+      <c r="D64" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G64" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H64" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I64" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J64" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K64" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -11796,13 +11121,6 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr"/>
-      <c r="E65" s="3" t="inlineStr"/>
-      <c r="F65" s="3" t="inlineStr">
-        <is>
           <t>### Analysis of the Provided Code
 The function `EC_GROUP_new_from_ecparameters` is responsible for creating an `EC_GROUP` structure from explicit elliptic curve parameters. It performs a series of validations, conversions, and error checks to ensure the parameters are correctly processed and the resulting `EC_GROUP` is valid.
 ---
@@ -11848,11 +11166,11 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D65" s="3" t="inlineStr"/>
+      <c r="E65" s="3" t="inlineStr"/>
+      <c r="F65" s="3" t="inlineStr"/>
       <c r="G65" s="3" t="inlineStr"/>
       <c r="H65" s="3" t="inlineStr"/>
-      <c r="I65" s="3" t="inlineStr"/>
-      <c r="J65" s="3" t="inlineStr"/>
-      <c r="K65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -11877,13 +11195,6 @@
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr"/>
-      <c r="E66" s="2" t="inlineStr"/>
-      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step to determine if there's a vulnerability.
 ### Code Snippet:
@@ -11927,19 +11238,19 @@
 **Note**: For a comprehensive security assessment, the surrounding code (e.g., variable declarations, the implementation of `pstmlist`, `pstm`, and `nl`) should also be examined.</t>
         </is>
       </c>
+      <c r="D66" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="G66" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H66" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I66" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J66" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K66" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -12012,21 +11323,6 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Tensorflow is an Open Source Machine Learning Framework. When building an XLA compilation cache, if default settings are used, TensorFlow triggers a null pointer dereference. In the default scenario, all devices are allowed, so `flr-&gt;config_proto` is `nullptr`. The fix will be included in TensorFlow 2.8.0. We will also cherrypick this commit on TensorFlow 2.7.1, TensorFlow 2.6.3, and TensorFlow 2.5.3, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Null Pointer Dereference in `device` Parameter:**
@@ -12041,19 +11337,19 @@
 The code contains vulnerabilities due to unchecked null pointers and lack of input validation, which could be exploited to cause crashes or undefined behavior. Thus, the answer is **YES**.</t>
         </is>
       </c>
+      <c r="D67" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="G67" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H67" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I67" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J67" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K67" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -12091,13 +11387,6 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr"/>
-      <c r="E68" s="3" t="inlineStr"/>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Function Purpose:** The function `clone_private_mount` creates a private clone of a mount structure based on the provided `path`. It involves checking the validity of the mount and its properties before cloning.
@@ -12114,11 +11403,11 @@
 **Result:** YES (Vulnerability detected due to potential NULL pointer dereference).</t>
         </is>
       </c>
+      <c r="D68" s="3" t="inlineStr"/>
+      <c r="E68" s="3" t="inlineStr"/>
+      <c r="F68" s="3" t="inlineStr"/>
       <c r="G68" s="3" t="inlineStr"/>
       <c r="H68" s="3" t="inlineStr"/>
-      <c r="I68" s="3" t="inlineStr"/>
-      <c r="J68" s="3" t="inlineStr"/>
-      <c r="K68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -12184,21 +11473,6 @@
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-125']</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>Tensorflow is an Open Source Machine Learning Framework. TensorFlow's type inference can cause a heap out of bounds read as the bounds checking is done in a `DCHECK` (which is a no-op during production). An attacker can control the `input_idx` variable such that `ix` would be larger than the number of values in `node_t.args`. The fix will be included in TensorFlow 2.8.0. This is the only affected version.</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 **Code Overview**
@@ -12237,19 +11511,19 @@
 3. **Error Handling:** Consider more explicit error handling and logging for incomplete or invalid types to avoid silent failures.</t>
         </is>
       </c>
+      <c r="D69" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="G69" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H69" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="I69" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J69" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K69" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -12359,13 +11633,6 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr"/>
-      <c r="E70" s="3" t="inlineStr"/>
-      <c r="F70" s="3" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Analysis:**
 1. **Input Validation:**
@@ -12388,11 +11655,11 @@
 **Answer:** NO</t>
         </is>
       </c>
+      <c r="D70" s="3" t="inlineStr"/>
+      <c r="E70" s="3" t="inlineStr"/>
+      <c r="F70" s="3" t="inlineStr"/>
       <c r="G70" s="3" t="inlineStr"/>
       <c r="H70" s="3" t="inlineStr"/>
-      <c r="I70" s="3" t="inlineStr"/>
-      <c r="J70" s="3" t="inlineStr"/>
-      <c r="K70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -12538,21 +11805,6 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>scheme/webauthn.c in Glewlwyd SSO server through 2.5.3 has a buffer overflow during FIDO2 signature validation in webauthn registration.</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 ### 1. **Code Overview**
 The provided code is a C function named `check_attestation_fido_u2f`, which appears to be part of a security protocol, likely related to FIDO U2F (Fast Identity Online Universal 2nd Factor) authentication. It performs various security checks, including certificate validation and signature verification.
@@ -12575,19 +11827,19 @@
 - **Review Error Logging**: Ensure that error logs do not inadvertently expose sensitive information.</t>
         </is>
       </c>
+      <c r="D71" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="G71" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H71" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="I71" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J71" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K71" s="2" t="inlineStr">
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -12940,13 +12192,6 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr"/>
-      <c r="E72" s="2" t="inlineStr"/>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 1. **Code Overview**:
 	* The provided code is a function `parse_command_modifiers` written in C, which appears to be part of the Vim text editor's source code.
@@ -12968,19 +12213,19 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D72" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G72" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H72" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="I72" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J72" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K72" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -13045,13 +12290,6 @@
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D73" s="3" t="inlineStr"/>
-      <c r="E73" s="3" t="inlineStr"/>
-      <c r="F73" s="3" t="inlineStr">
         <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Analysis:**
@@ -13075,11 +12313,11 @@
 Answer: (2) NO: No vulnerability.</t>
         </is>
       </c>
+      <c r="D73" s="3" t="inlineStr"/>
+      <c r="E73" s="3" t="inlineStr"/>
+      <c r="F73" s="3" t="inlineStr"/>
       <c r="G73" s="3" t="inlineStr"/>
       <c r="H73" s="3" t="inlineStr"/>
-      <c r="I73" s="3" t="inlineStr"/>
-      <c r="J73" s="3" t="inlineStr"/>
-      <c r="K73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -13140,13 +12378,6 @@
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D74" s="3" t="inlineStr"/>
-      <c r="E74" s="3" t="inlineStr"/>
-      <c r="F74" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 **Code Overview**
@@ -13179,11 +12410,11 @@
 **Note**: This analysis is based solely on the provided code snippet. The overall security of the system also depends on the correctness and security of the surrounding code, which is not analyzed here.</t>
         </is>
       </c>
+      <c r="D74" s="3" t="inlineStr"/>
+      <c r="E74" s="3" t="inlineStr"/>
+      <c r="F74" s="3" t="inlineStr"/>
       <c r="G74" s="3" t="inlineStr"/>
       <c r="H74" s="3" t="inlineStr"/>
-      <c r="I74" s="3" t="inlineStr"/>
-      <c r="J74" s="3" t="inlineStr"/>
-      <c r="K74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -13411,21 +12642,6 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-703']</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>TensorFlow is an open source platform for machine learning. Prior to versions 2.9.0, 2.8.1, 2.7.2, and 2.6.4, the implementation of `tf.raw_ops.LoadAndRemapMatrix does not fully validate the input arguments. This results in a `CHECK`-failure which can be used to trigger a denial of service attack. The code assumes `initializing_values` is a vector but there is no validation for this before accessing its value. Versions 2.9.0, 2.8.1, 2.7.2, and 2.6.4 contain a patch for this issue.</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Loop Variable Overflow Vulnerability:**
@@ -13448,19 +12664,19 @@
 **Conclusion:** The code contains a vulnerability due to the use of an `int` loop variable for iterating over potentially large tensor dimensions, leading to integer overflow and undefined behavior.</t>
         </is>
       </c>
+      <c r="D75" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G75" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H75" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I75" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J75" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K75" s="2" t="inlineStr">
+      <c r="H75" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -13608,13 +12824,6 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="inlineStr"/>
-      <c r="E76" s="3" t="inlineStr"/>
-      <c r="F76" s="3" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Analysis:**
 1. **Buffer Handling:**
@@ -13634,11 +12843,11 @@
 **Conclusion:** The code carefully manages buffer sizes, validates lengths, and handles edge cases (e.g., truncation, multibyte characters), eliminating common vulnerabilities like buffer overflows or format string attacks. No exploitable issues are detected.</t>
         </is>
       </c>
+      <c r="D76" s="3" t="inlineStr"/>
+      <c r="E76" s="3" t="inlineStr"/>
+      <c r="F76" s="3" t="inlineStr"/>
       <c r="G76" s="3" t="inlineStr"/>
       <c r="H76" s="3" t="inlineStr"/>
-      <c r="I76" s="3" t="inlineStr"/>
-      <c r="J76" s="3" t="inlineStr"/>
-      <c r="K76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
@@ -13686,21 +12895,6 @@
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-617']</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t>Tensorflow is an Open Source Machine Learning Framework. The Grappler optimizer in TensorFlow can be used to cause a denial of service by altering a `SavedModel` such that `SafeToRemoveIdentity` would trigger `CHECK` failures. The fix will be included in TensorFlow 2.8.0. We will also cherrypick this commit on TensorFlow 2.7.1, TensorFlow 2.6.3, and TensorFlow 2.5.3, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F77" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step to determine if there's a vulnerability.
 **Code Overview**
@@ -13737,11 +12931,11 @@
 However, it's worth noting the robustness issue for the developers to address.</t>
         </is>
       </c>
+      <c r="D77" s="3" t="inlineStr"/>
+      <c r="E77" s="3" t="inlineStr"/>
+      <c r="F77" s="3" t="inlineStr"/>
       <c r="G77" s="3" t="inlineStr"/>
       <c r="H77" s="3" t="inlineStr"/>
-      <c r="I77" s="3" t="inlineStr"/>
-      <c r="J77" s="3" t="inlineStr"/>
-      <c r="K77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
@@ -13784,21 +12978,6 @@
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="inlineStr">
-        <is>
-          <t>A NULL pointer dereference flaw in diFree in fs/jfs/inode.c in Journaled File System (JFS)in the Linux kernel. This could allow a local attacker to crash the system or leak kernel internal information.</t>
-        </is>
-      </c>
-      <c r="F78" s="3" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Analysis:**
 1. **Function Purpose**: The `jfs_evict_inode` function handles inode eviction in the JFS filesystem, cleaning up resources like page caches, disk quotas, and allocation group tracking.
@@ -13818,11 +12997,11 @@
 **Result**: NO.</t>
         </is>
       </c>
+      <c r="D78" s="3" t="inlineStr"/>
+      <c r="E78" s="3" t="inlineStr"/>
+      <c r="F78" s="3" t="inlineStr"/>
       <c r="G78" s="3" t="inlineStr"/>
       <c r="H78" s="3" t="inlineStr"/>
-      <c r="I78" s="3" t="inlineStr"/>
-      <c r="J78" s="3" t="inlineStr"/>
-      <c r="K78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
@@ -13982,21 +13161,6 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="inlineStr">
-        <is>
-          <t>TensorFlow is an open source platform for machine learning. Prior to versions 2.9.0, 2.8.1, 2.7.2, and 2.6.4, the implementation of `tf.raw_ops.EditDistance` has incomplete validation. Users can pass negative values to cause a segmentation fault based denial of service. In multiple places throughout the code, one may compute an index for a write operation. However, the existing validation only checks against the upper bound of the array. Hence, it is possible to write before the array by massaging the input to generate negative values for `loc`. Versions 2.9.0, 2.8.1, 2.7.2, and 2.6.4 contain a patch for this issue.</t>
-        </is>
-      </c>
-      <c r="F79" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 ### 1. **Input Validation**
 - The code uses `OP_REQUIRES_OK` to check the return status of input retrieval operations, which is good for error handling.
@@ -14032,11 +13196,11 @@
 - Verify the implementation of `ValidateShapes` and `sparse::Group` to ensure they meet the assumed standards for robustness and security.</t>
         </is>
       </c>
+      <c r="D79" s="3" t="inlineStr"/>
+      <c r="E79" s="3" t="inlineStr"/>
+      <c r="F79" s="3" t="inlineStr"/>
       <c r="G79" s="3" t="inlineStr"/>
       <c r="H79" s="3" t="inlineStr"/>
-      <c r="I79" s="3" t="inlineStr"/>
-      <c r="J79" s="3" t="inlineStr"/>
-      <c r="K79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
@@ -14085,21 +13249,6 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-617']</t>
-        </is>
-      </c>
-      <c r="E80" s="3" t="inlineStr">
-        <is>
-          <t>Tensorflow is an Open Source Machine Learning Framework. The Grappler optimizer in TensorFlow can be used to cause a denial of service by altering a `SavedModel` such that `SafeToRemoveIdentity` would trigger `CHECK` failures. The fix will be included in TensorFlow 2.8.0. We will also cherrypick this commit on TensorFlow 2.7.1, TensorFlow 2.6.3, and TensorFlow 2.5.3, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F80" s="3" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Analysis:**
 1. **Function Purpose:** The function `SafeToRemoveIdentity` determines whether an identity node in a computation graph can be safely removed during optimization. It checks multiple conditions to ensure removal does not break the graph's correctness.
@@ -14123,11 +13272,11 @@
 Answer: (2) NO: No vulnerability.</t>
         </is>
       </c>
+      <c r="D80" s="3" t="inlineStr"/>
+      <c r="E80" s="3" t="inlineStr"/>
+      <c r="F80" s="3" t="inlineStr"/>
       <c r="G80" s="3" t="inlineStr"/>
       <c r="H80" s="3" t="inlineStr"/>
-      <c r="I80" s="3" t="inlineStr"/>
-      <c r="J80" s="3" t="inlineStr"/>
-      <c r="K80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
@@ -14226,21 +13375,6 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-125']</t>
-        </is>
-      </c>
-      <c r="E81" s="3" t="inlineStr">
-        <is>
-          <t>An out-of-bounds read flaw was found in the Linux kernel’s io_uring module in the way a user triggers the io_read() function with some special parameters. This flaw allows a local user to read some memory out of bounds.</t>
-        </is>
-      </c>
-      <c r="F81" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
 The `io_read` function appears to be part of a Linux kernel I/O subsystem, specifically handling read operations for the io_uring asynchronous I/O interface. It manages various aspects of the read operation, including setting up the I/O vector, handling synchronous and asynchronous read paths, and managing retries.
@@ -14272,11 +13406,11 @@
 - Ensure that input size validation is sufficiently robust to prevent potential denial-of-service (DoS) scenarios.</t>
         </is>
       </c>
+      <c r="D81" s="3" t="inlineStr"/>
+      <c r="E81" s="3" t="inlineStr"/>
+      <c r="F81" s="3" t="inlineStr"/>
       <c r="G81" s="3" t="inlineStr"/>
       <c r="H81" s="3" t="inlineStr"/>
-      <c r="I81" s="3" t="inlineStr"/>
-      <c r="J81" s="3" t="inlineStr"/>
-      <c r="K81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n">
@@ -14323,13 +13457,6 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr"/>
-      <c r="E82" s="3" t="inlineStr"/>
-      <c r="F82" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
 The function `sctp_make_strreset_req` is responsible for creating an SCTP (Stream Control Transmission Protocol) chunk for a stream reset request. It takes parameters related to an SCTP association, stream numbers, and flags indicating whether to include out and/or in reset requests.
@@ -14349,11 +13476,11 @@
 **Reasoning**: The lack of input validation for `asoc` and `stream_list` (when `stream_num &gt; 0`) poses a risk of null pointer dereference or memory corruption, which are considered vulnerabilities. Additionally, the incomplete error handling could lead to unexpected behavior in case of failures from `sctp_addto_chunk` or other underlying functions. These issues warrant a "YES" for vulnerability detected, assuming the context allows these flaws to be exploitable.</t>
         </is>
       </c>
+      <c r="D82" s="3" t="inlineStr"/>
+      <c r="E82" s="3" t="inlineStr"/>
+      <c r="F82" s="3" t="inlineStr"/>
       <c r="G82" s="3" t="inlineStr"/>
       <c r="H82" s="3" t="inlineStr"/>
-      <c r="I82" s="3" t="inlineStr"/>
-      <c r="J82" s="3" t="inlineStr"/>
-      <c r="K82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -14567,13 +13694,6 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr"/>
-      <c r="E83" s="2" t="inlineStr"/>
-      <c r="F83" s="2" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 ### 1. **Function Overview**
 The provided function, `pjmedia_rtcp_xr_rx_rtcp_xr`, appears to be part of a media library (likely PJSIP) handling the reception of RTCP-XR (RTP Control Protocol for XML - Extended Reports) packets. It processes various report blocks within an RTCP packet.
@@ -14598,19 +13718,19 @@
 **Note**: This analysis is limited to the provided code snippet. The overall security of the system or library also depends on factors outside this function, such as input validation at higher levels, secure memory management practices, and the context in which the processed data is used.</t>
         </is>
       </c>
+      <c r="D83" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G83" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H83" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I83" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J83" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K83" s="2" t="inlineStr">
+      <c r="H83" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -15078,21 +14198,6 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D84" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E84" s="3" t="inlineStr">
-        <is>
-          <t>GPAC 2.1-DEV-rev87-g053aae8-master. has a Null Pointer Dereference vulnerability in gf_isom_parse_movie_boxes_internal due to improper return value handling of GF_SKIP_BOX, which causes a Denial of Service. This vulnerability was fixed in commit 37592ad.</t>
-        </is>
-      </c>
-      <c r="F84" s="3" t="inlineStr">
-        <is>
           <t>After a thorough analysis of the provided code, the function `gf_isom_parse_movie_boxes_internal` appears to be a robust implementation of an ISO/MP4 file parser. The code handles various box types, manages memory allocation and deallocation carefully, checks for errors, and ensures that critical boxes like `MOOV` and `META` are present. Key observations include:
 1. **Error Handling**: The function checks return values from parsing and list operations, returning appropriate errors when issues arise (e.g., memory allocation failures, duplicate boxes, missing required boxes).
 2. **Memory Management**: Boxes are either added to the appropriate list or explicitly deleted (`gf_isom_box_del`) to prevent memory leaks. For example, duplicate boxes (like `MOOV`, `META`, `FTYP`) are deleted immediately upon detection.
@@ -15104,11 +14209,11 @@
 **Answer:** NO</t>
         </is>
       </c>
+      <c r="D84" s="3" t="inlineStr"/>
+      <c r="E84" s="3" t="inlineStr"/>
+      <c r="F84" s="3" t="inlineStr"/>
       <c r="G84" s="3" t="inlineStr"/>
       <c r="H84" s="3" t="inlineStr"/>
-      <c r="I84" s="3" t="inlineStr"/>
-      <c r="J84" s="3" t="inlineStr"/>
-      <c r="K84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
@@ -15229,21 +14334,6 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-189']</t>
-        </is>
-      </c>
-      <c r="E85" s="3" t="inlineStr">
-        <is>
-          <t>Multiple integer overflows in the read_bitmap_file_data function in io-xbm.c in gdk-pixbuf before 2.26.1 allow remote attackers to cause a denial of service (application crash) via a negative (1) height or (2) width in an XBM file, which triggers a heap-based buffer overflow.</t>
-        </is>
-      </c>
-      <c r="F85" s="3" t="inlineStr">
-        <is>
           <t>YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Integer Overflow in Size Calculation:**
@@ -15260,11 +14350,11 @@
 **Conclusion:** The code is vulnerable due to an unchecked integer overflow in the calculation of the buffer size, leading to a potential heap-based buffer overflow.</t>
         </is>
       </c>
+      <c r="D85" s="3" t="inlineStr"/>
+      <c r="E85" s="3" t="inlineStr"/>
+      <c r="F85" s="3" t="inlineStr"/>
       <c r="G85" s="3" t="inlineStr"/>
       <c r="H85" s="3" t="inlineStr"/>
-      <c r="I85" s="3" t="inlineStr"/>
-      <c r="J85" s="3" t="inlineStr"/>
-      <c r="K85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -15312,21 +14402,6 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-369']</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>In Deark before v1.5.8, a specially crafted input file can cause a division by zero in (src/fmtutil.c) because of the value of pixelsize.</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Division by Zero Vulnerability:**
@@ -15340,19 +14415,19 @@
 **Conclusion:** The division by zero vulnerability is sufficient to classify the code as vulnerable. The lack of input validation and error checking for buffer bounds exacerbates the issue.</t>
         </is>
       </c>
+      <c r="D86" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="G86" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H86" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I86" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J86" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K86" s="2" t="inlineStr">
+      <c r="H86" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -15371,21 +14446,6 @@
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E87" s="3" t="inlineStr">
-        <is>
-          <t>fs/seq_file.c in the Linux kernel 3.16 through 5.13.x before 5.13.4 does not properly restrict seq buffer allocations, leading to an integer overflow, an Out-of-bounds Write, and escalation to root by an unprivileged user, aka CID-8cae8cd89f05.</t>
-        </is>
-      </c>
-      <c r="F87" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step to determine if it contains a vulnerability.
 ### Code Snippet:
@@ -15416,11 +14476,11 @@
 **Note:** This assessment is limited to the code snippet provided and assumes proper error handling, input validation, and memory management practices are implemented in the surrounding code.</t>
         </is>
       </c>
+      <c r="D87" s="3" t="inlineStr"/>
+      <c r="E87" s="3" t="inlineStr"/>
+      <c r="F87" s="3" t="inlineStr"/>
       <c r="G87" s="3" t="inlineStr"/>
       <c r="H87" s="3" t="inlineStr"/>
-      <c r="I87" s="3" t="inlineStr"/>
-      <c r="J87" s="3" t="inlineStr"/>
-      <c r="K87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n">
@@ -15884,21 +14944,6 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D88" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E88" s="3" t="inlineStr">
-        <is>
-          <t>GPAC 2.1-DEV-rev87-g053aae8-master. has a Null Pointer Dereference vulnerability in gf_isom_parse_movie_boxes_internal due to improper return value handling of GF_SKIP_BOX, which causes a Denial of Service. This vulnerability was fixed in commit 37592ad.</t>
-        </is>
-      </c>
-      <c r="F88" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 Given the complexity of the provided code, I'll break down the analysis into manageable steps to determine if a vulnerability is present.
 ### **1. Code Overview**
@@ -15931,11 +14976,11 @@
 **Note**: This analysis is limited to the provided code snippet and focuses on common vulnerability categories. A comprehensive security audit would require reviewing the entire project, including all dependent functions and the specific deployment environment.</t>
         </is>
       </c>
+      <c r="D88" s="3" t="inlineStr"/>
+      <c r="E88" s="3" t="inlineStr"/>
+      <c r="F88" s="3" t="inlineStr"/>
       <c r="G88" s="3" t="inlineStr"/>
       <c r="H88" s="3" t="inlineStr"/>
-      <c r="I88" s="3" t="inlineStr"/>
-      <c r="J88" s="3" t="inlineStr"/>
-      <c r="K88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n">
@@ -16053,13 +15098,6 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D89" s="3" t="inlineStr"/>
-      <c r="E89" s="3" t="inlineStr"/>
-      <c r="F89" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 ### 1. **Buffer Definition and Usage**
 - **Buffer Size**: The buffer is defined with `sizeof(squashfs_dir_entry_2) + SQUASHFS_NAME_LEN + 1`, which seems to account for the structure and the maximum possible name length plus a null terminator. This suggests an attempt to prevent buffer overflows related to name storage.
@@ -16081,11 +15119,11 @@
 **Note**: This analysis is based on the provided code snippet. A comprehensive security audit would require examining the entire codebase, including functions like `check_name`, `read_inode`, `lookup_entry`, and the definitions of structures and macros used.</t>
         </is>
       </c>
+      <c r="D89" s="3" t="inlineStr"/>
+      <c r="E89" s="3" t="inlineStr"/>
+      <c r="F89" s="3" t="inlineStr"/>
       <c r="G89" s="3" t="inlineStr"/>
       <c r="H89" s="3" t="inlineStr"/>
-      <c r="I89" s="3" t="inlineStr"/>
-      <c r="J89" s="3" t="inlineStr"/>
-      <c r="K89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n">
@@ -16135,21 +15173,6 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D90" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E90" s="3" t="inlineStr">
-        <is>
-          <t>mruby is vulnerable to NULL Pointer Dereference</t>
-        </is>
-      </c>
-      <c r="F90" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step to determine if there's a vulnerability.
 **Code Overview**
 The code is a function `mrb_ary_shift_m` which appears to be part of the Mr. Ruby (MRB) implementation, specifically handling the `shift` method for arrays. The `shift` method removes elements from the beginning of an array. The function takes an optional argument `n` to remove multiple elements at once.
@@ -16178,11 +15201,11 @@
 **Result: (2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D90" s="3" t="inlineStr"/>
+      <c r="E90" s="3" t="inlineStr"/>
+      <c r="F90" s="3" t="inlineStr"/>
       <c r="G90" s="3" t="inlineStr"/>
       <c r="H90" s="3" t="inlineStr"/>
-      <c r="I90" s="3" t="inlineStr"/>
-      <c r="J90" s="3" t="inlineStr"/>
-      <c r="K90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n">
@@ -16593,13 +15616,6 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="inlineStr"/>
-      <c r="E91" s="3" t="inlineStr"/>
-      <c r="F91" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 1. **Code Overview**:
 	* The provided code is a C function `cp_create` that initializes and configures various parameters for image encoding (likely JPEG 2000 based on the context).
@@ -16634,11 +15650,11 @@
 The provided code snippet exhibits robust memory management, thorough input validation, safe arithmetic operations, and consistent error handling, indicating no apparent vulnerabilities based on the given analysis.</t>
         </is>
       </c>
+      <c r="D91" s="3" t="inlineStr"/>
+      <c r="E91" s="3" t="inlineStr"/>
+      <c r="F91" s="3" t="inlineStr"/>
       <c r="G91" s="3" t="inlineStr"/>
       <c r="H91" s="3" t="inlineStr"/>
-      <c r="I91" s="3" t="inlineStr"/>
-      <c r="J91" s="3" t="inlineStr"/>
-      <c r="K91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n">
@@ -16951,21 +15967,6 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-125']</t>
-        </is>
-      </c>
-      <c r="E92" s="3" t="inlineStr">
-        <is>
-          <t>Out-of-bounds Read in GitHub repository radareorg/radare2 prior to 5.7.0.</t>
-        </is>
-      </c>
-      <c r="F92" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 ### 1. **Function Overview**
 The provided function, `string_scan_range`, appears to be part of a binary analysis tool, likely Radare2, given the `R` prefixes and the context. It scans a specified range within a binary file for strings, attempting to detect and handle various string types (ASCII, UTF-8, Wide, Wide32).
@@ -16987,11 +15988,11 @@
 **Result: (2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D92" s="3" t="inlineStr"/>
+      <c r="E92" s="3" t="inlineStr"/>
+      <c r="F92" s="3" t="inlineStr"/>
       <c r="G92" s="3" t="inlineStr"/>
       <c r="H92" s="3" t="inlineStr"/>
-      <c r="I92" s="3" t="inlineStr"/>
-      <c r="J92" s="3" t="inlineStr"/>
-      <c r="K92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n">
@@ -17303,13 +16304,6 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D93" s="3" t="inlineStr"/>
-      <c r="E93" s="3" t="inlineStr"/>
-      <c r="F93" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 ### 1. **Input Validation**
 The function `load` reads data from a file (`XModuleBase&amp; f`). Initial checks are performed on the number of instruments, patterns, and channels, but these are more about resource allocation than input validation.
@@ -17339,11 +16333,11 @@
 - Review the `orders` array handling to prevent potential overflows.</t>
         </is>
       </c>
+      <c r="D93" s="3" t="inlineStr"/>
+      <c r="E93" s="3" t="inlineStr"/>
+      <c r="F93" s="3" t="inlineStr"/>
       <c r="G93" s="3" t="inlineStr"/>
       <c r="H93" s="3" t="inlineStr"/>
-      <c r="I93" s="3" t="inlineStr"/>
-      <c r="J93" s="3" t="inlineStr"/>
-      <c r="K93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n">
@@ -17405,13 +16399,6 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D94" s="3" t="inlineStr"/>
-      <c r="E94" s="3" t="inlineStr"/>
-      <c r="F94" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 **Code Overview**
 ----------------
@@ -17447,11 +16434,11 @@
 **Answer**: **YES** (Vulnerability detected, related to potential memory exhaustion)</t>
         </is>
       </c>
+      <c r="D94" s="3" t="inlineStr"/>
+      <c r="E94" s="3" t="inlineStr"/>
+      <c r="F94" s="3" t="inlineStr"/>
       <c r="G94" s="3" t="inlineStr"/>
       <c r="H94" s="3" t="inlineStr"/>
-      <c r="I94" s="3" t="inlineStr"/>
-      <c r="J94" s="3" t="inlineStr"/>
-      <c r="K94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
@@ -17568,21 +16555,6 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D95" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-120']</t>
-        </is>
-      </c>
-      <c r="E95" s="3" t="inlineStr">
-        <is>
-          <t>A buffer overflow vulnerability in jetp3852_print_page() in devices/gdev3852.c of Artifex Software GhostScript v9.50 allows a remote attacker to escalate privileges via a crafted PDF file. This is fixed in v9.51.</t>
-        </is>
-      </c>
-      <c r="F95" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
 The function `jetp3852_print_page` appears to be part of a printer driver, specifically for handling the printing of a page to a JetDirect (HP JetDirect printer) device. It takes a device context (`pdev`) and a print stream (`prn_stream`) as inputs. The function's primary tasks include:
@@ -17611,11 +16583,11 @@
 - If this function is part of a larger codebase, ensure that inputs from external sources are properly validated and sanitized before being used within this function.</t>
         </is>
       </c>
+      <c r="D95" s="3" t="inlineStr"/>
+      <c r="E95" s="3" t="inlineStr"/>
+      <c r="F95" s="3" t="inlineStr"/>
       <c r="G95" s="3" t="inlineStr"/>
       <c r="H95" s="3" t="inlineStr"/>
-      <c r="I95" s="3" t="inlineStr"/>
-      <c r="J95" s="3" t="inlineStr"/>
-      <c r="K95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n">
@@ -17652,21 +16624,6 @@
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-416']</t>
-        </is>
-      </c>
-      <c r="E96" s="3" t="inlineStr">
-        <is>
-          <t>TensorFlow is an end-to-end open source platform for machine learning. In affected versions the implementation for `tf.raw_ops.BoostedTreesCreateEnsemble` can result in a use after free error if an attacker supplies specially crafted arguments. The [implementation](https://github.com/tensorflow/tensorflow/blob/f24faa153ad31a4b51578f8181d3aaab77a1ddeb/tensorflow/core/kernels/boosted_trees/resource_ops.cc#L55) uses a reference counted resource and decrements the refcount if the initialization fails, as it should. However, when the code was written, the resource was represented as a naked pointer but later refactoring has changed it to be a smart pointer. Thus, when the pointer leaves the scope, a subsequent `free`-ing of the resource occurs, but this fails to take into account that the refcount has already reached 0, thus the resource has been already freed. During this double-free process, members of the resource object are accessed for cleanup but they are invalid as the entire resource has been freed. We have patched the issue in GitHub commit 5ecec9c6fbdbc6be03295685190a45e7eee726ab. The fix will be included in TensorFlow 2.6.0. We will also cherrypick this commit on TensorFlow 2.5.1, TensorFlow 2.4.3, and TensorFlow 2.3.4, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F96" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step from a **static program analysis** and **security** perspective.
 ---
@@ -17744,11 +16701,11 @@
 &gt; **Reason**: The manual call to `result-&gt;Unref()` on a `unique_ptr`-managed object may lead to a **double-free** or **use-after-free** if `Unref()` affects the object's lifetime or validity. This is a **memory safety issue** and a potential security vulnerability.</t>
         </is>
       </c>
+      <c r="D96" s="3" t="inlineStr"/>
+      <c r="E96" s="3" t="inlineStr"/>
+      <c r="F96" s="3" t="inlineStr"/>
       <c r="G96" s="3" t="inlineStr"/>
       <c r="H96" s="3" t="inlineStr"/>
-      <c r="I96" s="3" t="inlineStr"/>
-      <c r="J96" s="3" t="inlineStr"/>
-      <c r="K96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n">
@@ -17844,13 +16801,6 @@
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D97" s="3" t="inlineStr"/>
-      <c r="E97" s="3" t="inlineStr"/>
-      <c r="F97" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step from a **static program analysis** and **security** perspective.
 ---
@@ -17957,11 +16907,11 @@
 **(1) YES: Vulnerability detected.**</t>
         </is>
       </c>
+      <c r="D97" s="3" t="inlineStr"/>
+      <c r="E97" s="3" t="inlineStr"/>
+      <c r="F97" s="3" t="inlineStr"/>
       <c r="G97" s="3" t="inlineStr"/>
       <c r="H97" s="3" t="inlineStr"/>
-      <c r="I97" s="3" t="inlineStr"/>
-      <c r="J97" s="3" t="inlineStr"/>
-      <c r="K97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n">
@@ -18074,21 +17024,6 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D98" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-369']</t>
-        </is>
-      </c>
-      <c r="E98" s="3" t="inlineStr">
-        <is>
-          <t>Tensorflow is an Open Source Machine Learning Framework. The implementation of `FractionalMaxPool` can be made to crash a TensorFlow process via a division by 0. The fix will be included in TensorFlow 2.8.0. We will also cherrypick this commit on TensorFlow 2.7.1, TensorFlow 2.6.3, and TensorFlow 2.5.3, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F98" s="3" t="inlineStr">
-        <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Explanation:**
 1. **Input Validation:** The code checks that the input tensor is 4-dimensional using `OP_REQUIRES`, ensuring the expected input structure.
@@ -18102,11 +17037,11 @@
 **Conclusion:** The code properly validates inputs, handles edge cases (e.g., clamping indices), and uses TensorFlow's error-handling mechanisms to manage allocation failures. No direct vulnerabilities (e.g., buffer overflows, use-after-free, or unchecked inputs leading to crashes) are present in the provided code.</t>
         </is>
       </c>
+      <c r="D98" s="3" t="inlineStr"/>
+      <c r="E98" s="3" t="inlineStr"/>
+      <c r="F98" s="3" t="inlineStr"/>
       <c r="G98" s="3" t="inlineStr"/>
       <c r="H98" s="3" t="inlineStr"/>
-      <c r="I98" s="3" t="inlineStr"/>
-      <c r="J98" s="3" t="inlineStr"/>
-      <c r="K98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n">
@@ -18178,13 +17113,6 @@
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D99" s="3" t="inlineStr"/>
-      <c r="E99" s="3" t="inlineStr"/>
-      <c r="F99" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
@@ -18224,11 +17152,11 @@
 ```</t>
         </is>
       </c>
+      <c r="D99" s="3" t="inlineStr"/>
+      <c r="E99" s="3" t="inlineStr"/>
+      <c r="F99" s="3" t="inlineStr"/>
       <c r="G99" s="3" t="inlineStr"/>
       <c r="H99" s="3" t="inlineStr"/>
-      <c r="I99" s="3" t="inlineStr"/>
-      <c r="J99" s="3" t="inlineStr"/>
-      <c r="K99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n">
@@ -18426,13 +17354,6 @@
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D100" s="3" t="inlineStr"/>
-      <c r="E100" s="3" t="inlineStr"/>
-      <c r="F100" s="3" t="inlineStr">
-        <is>
           <t>YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Memory Allocation with Negative Size:**
@@ -18447,11 +17368,11 @@
 **Conclusion:** The code contains a vulnerability due to improper validation of the allocation size, which can lead to memory corruption. This is a critical issue that requires fixing by adding checks to ensure `i` is non-negative before allocation.</t>
         </is>
       </c>
+      <c r="D100" s="3" t="inlineStr"/>
+      <c r="E100" s="3" t="inlineStr"/>
+      <c r="F100" s="3" t="inlineStr"/>
       <c r="G100" s="3" t="inlineStr"/>
       <c r="H100" s="3" t="inlineStr"/>
-      <c r="I100" s="3" t="inlineStr"/>
-      <c r="J100" s="3" t="inlineStr"/>
-      <c r="K100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n">
@@ -18504,21 +17425,6 @@
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E101" s="3" t="inlineStr">
-        <is>
-          <t>An issue was discovered in the Linux kernel through 5.16-rc6. There is a lack of check after calling vzalloc() and lack of free after allocation in drivers/media/test-drivers/vidtv/vidtv_s302m.c.</t>
-        </is>
-      </c>
-      <c r="F101" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step from a **static program analysis** and **security** perspective.
 ---
@@ -18590,11 +17496,11 @@
 &gt; **Reason**: Lack of validation on `args.name`, `args.src_buf`, `args.src_buf_sz`, and `args.head` could lead to memory corruption or denial of service if these inputs are attacker-controlled.</t>
         </is>
       </c>
+      <c r="D101" s="3" t="inlineStr"/>
+      <c r="E101" s="3" t="inlineStr"/>
+      <c r="F101" s="3" t="inlineStr"/>
       <c r="G101" s="3" t="inlineStr"/>
       <c r="H101" s="3" t="inlineStr"/>
-      <c r="I101" s="3" t="inlineStr"/>
-      <c r="J101" s="3" t="inlineStr"/>
-      <c r="K101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n">
@@ -18621,21 +17527,6 @@
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D102" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E102" s="3" t="inlineStr">
-        <is>
-          <t>Buffer overflow in the send_control_msg function in hw/char/virtio-serial-bus.c in QEMU before 2.4.0 allows guest users to cause a denial of service (QEMU process crash) via a crafted virtio control message.</t>
-        </is>
-      </c>
-      <c r="F102" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 **Code Snippet Analysis**
@@ -18690,11 +17581,11 @@
 ```</t>
         </is>
       </c>
+      <c r="D102" s="3" t="inlineStr"/>
+      <c r="E102" s="3" t="inlineStr"/>
+      <c r="F102" s="3" t="inlineStr"/>
       <c r="G102" s="3" t="inlineStr"/>
       <c r="H102" s="3" t="inlineStr"/>
-      <c r="I102" s="3" t="inlineStr"/>
-      <c r="J102" s="3" t="inlineStr"/>
-      <c r="K102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n">
@@ -19007,21 +17898,6 @@
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D103" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-125']</t>
-        </is>
-      </c>
-      <c r="E103" s="3" t="inlineStr">
-        <is>
-          <t>Out-of-bounds Read in GitHub repository radareorg/radare2 prior to 5.7.0.</t>
-        </is>
-      </c>
-      <c r="F103" s="3" t="inlineStr">
-        <is>
           <t>NO: No vulnerability.
 The code for `string_scan_range` appears to handle memory allocations and buffer operations safely. Key points include:
 1. **Memory Allocation Checks**: The function checks that the range length (`len = to - from`) is within valid bounds (1 to ST32_MAX), preventing excessively large allocations that could lead to memory exhaustion or overflow.
@@ -19034,11 +17910,11 @@
 **Answer:** NO</t>
         </is>
       </c>
+      <c r="D103" s="3" t="inlineStr"/>
+      <c r="E103" s="3" t="inlineStr"/>
+      <c r="F103" s="3" t="inlineStr"/>
       <c r="G103" s="3" t="inlineStr"/>
       <c r="H103" s="3" t="inlineStr"/>
-      <c r="I103" s="3" t="inlineStr"/>
-      <c r="J103" s="3" t="inlineStr"/>
-      <c r="K103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n">
@@ -19234,21 +18110,6 @@
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D104" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E104" s="3" t="inlineStr">
-        <is>
-          <t>Heap-based Buffer Overflow in GitHub repository vim/vim prior to 8.2.4436.</t>
-        </is>
-      </c>
-      <c r="F104" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 1. **Code Overview**:
 	* The provided code is a function `change_indent` written in C, likely part of the Vim text editor.
@@ -19282,11 +18143,11 @@
 3. **Code Review**: Perform a thorough code review of the entire function and related functions (`ml_get_curline()`, `shift_line()`, etc.) to ensure overall security and stability.</t>
         </is>
       </c>
+      <c r="D104" s="3" t="inlineStr"/>
+      <c r="E104" s="3" t="inlineStr"/>
+      <c r="F104" s="3" t="inlineStr"/>
       <c r="G104" s="3" t="inlineStr"/>
       <c r="H104" s="3" t="inlineStr"/>
-      <c r="I104" s="3" t="inlineStr"/>
-      <c r="J104" s="3" t="inlineStr"/>
-      <c r="K104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -19432,21 +18293,6 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>scheme/webauthn.c in Glewlwyd SSO server through 2.5.3 has a buffer overflow during FIDO2 signature validation in webauthn registration.</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr">
-        <is>
           <t>YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Buffer Overflow in `data_signed` Array:**
@@ -19461,19 +18307,19 @@
 Both vulnerabilities are critical. The buffer overflow is a direct memory safety issue, while the incorrect length calculation undermines the cryptographic verification process. These flaws could be exploited to bypass security checks or cause denial of service.</t>
         </is>
       </c>
+      <c r="D105" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E105" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F105" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="G105" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H105" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I105" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J105" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K105" s="2" t="inlineStr">
+      <c r="H105" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -19494,13 +18340,6 @@
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D106" s="3" t="inlineStr"/>
-      <c r="E106" s="3" t="inlineStr"/>
-      <c r="F106" s="3" t="inlineStr">
         <is>
           <t>(2) NO: No vulnerability.
 **Step-by-Step Explanation:**
@@ -19512,11 +18351,11 @@
 **Conclusion:** No vulnerabilities are present in the given code under standard assumptions. The answer is **NO**.</t>
         </is>
       </c>
+      <c r="D106" s="3" t="inlineStr"/>
+      <c r="E106" s="3" t="inlineStr"/>
+      <c r="F106" s="3" t="inlineStr"/>
       <c r="G106" s="3" t="inlineStr"/>
       <c r="H106" s="3" t="inlineStr"/>
-      <c r="I106" s="3" t="inlineStr"/>
-      <c r="J106" s="3" t="inlineStr"/>
-      <c r="K106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n">
@@ -19549,13 +18388,6 @@
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D107" s="3" t="inlineStr"/>
-      <c r="E107" s="3" t="inlineStr"/>
-      <c r="F107" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step from a static program analysis and security perspective.
 ---
@@ -19619,11 +18451,11 @@
 **Reason:** Missing NULL check on `old_mnt` after `real_mount()` can lead to NULL pointer dereference.</t>
         </is>
       </c>
+      <c r="D107" s="3" t="inlineStr"/>
+      <c r="E107" s="3" t="inlineStr"/>
+      <c r="F107" s="3" t="inlineStr"/>
       <c r="G107" s="3" t="inlineStr"/>
       <c r="H107" s="3" t="inlineStr"/>
-      <c r="I107" s="3" t="inlineStr"/>
-      <c r="J107" s="3" t="inlineStr"/>
-      <c r="K107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -19692,21 +18524,6 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E108" s="2" t="inlineStr">
-        <is>
-          <t>Tensorflow is an Open Source Machine Learning Framework. When building an XLA compilation cache, if default settings are used, TensorFlow triggers a null pointer dereference. In the default scenario, all devices are allowed, so `flr-&gt;config_proto` is `nullptr`. The fix will be included in TensorFlow 2.8.0. We will also cherrypick this commit on TensorFlow 2.7.1, TensorFlow 2.6.3, and TensorFlow 2.5.3, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Code Overview**
 The `BuildXlaCompilationCache` function initializes and returns an `XlaCompilationCache` object based on the provided `device`, `flr`, `platform_info`, and outputs it through the `cache` pointer. It involves interactions with XLA (Accelerated Linear Algebra) compilers, platform managers, and client options.
@@ -19735,19 +18552,19 @@
 **Reasoning**: Primarily due to the potential concurrency issue and the less-than-ideal error handling with `ValueOrDie()`, which could be exploitable or lead to service disruption in a multi-threaded production environment. The memory allocation point, while a concern, is more context-dependent and less clearly a vulnerability in modern systems.</t>
         </is>
       </c>
+      <c r="D108" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G108" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H108" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I108" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J108" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K108" s="2" t="inlineStr">
+      <c r="H108" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -19780,13 +18597,6 @@
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
-        <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D109" s="3" t="inlineStr"/>
-      <c r="E109" s="3" t="inlineStr"/>
-      <c r="F109" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 **Code Overview**
@@ -19816,11 +18626,11 @@
 **Mitigation Suggestion**: Add an explicit check at the beginning of the function to return an error (e.g., `-EBADF`) if `fd &lt; 0`.</t>
         </is>
       </c>
+      <c r="D109" s="3" t="inlineStr"/>
+      <c r="E109" s="3" t="inlineStr"/>
+      <c r="F109" s="3" t="inlineStr"/>
       <c r="G109" s="3" t="inlineStr"/>
       <c r="H109" s="3" t="inlineStr"/>
-      <c r="I109" s="3" t="inlineStr"/>
-      <c r="J109" s="3" t="inlineStr"/>
-      <c r="K109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n">
@@ -19862,21 +18672,6 @@
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D110" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E110" s="3" t="inlineStr">
-        <is>
-          <t>A NULL pointer dereference flaw in diFree in fs/jfs/inode.c in Journaled File System (JFS)in the Linux kernel. This could allow a local attacker to crash the system or leak kernel internal information.</t>
-        </is>
-      </c>
-      <c r="F110" s="3" t="inlineStr">
         <is>
           <t>Let's analyze the provided code step-by-step from a **static program analysis** and **security vulnerability detection** perspective.
 ---
@@ -19997,11 +18792,11 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D110" s="3" t="inlineStr"/>
+      <c r="E110" s="3" t="inlineStr"/>
+      <c r="F110" s="3" t="inlineStr"/>
       <c r="G110" s="3" t="inlineStr"/>
       <c r="H110" s="3" t="inlineStr"/>
-      <c r="I110" s="3" t="inlineStr"/>
-      <c r="J110" s="3" t="inlineStr"/>
-      <c r="K110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="3" t="n">
@@ -20155,13 +18950,6 @@
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D111" s="3" t="inlineStr"/>
-      <c r="E111" s="3" t="inlineStr"/>
-      <c r="F111" s="3" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Buffer Overflow in Run Mode Loop:**
@@ -20178,11 +18966,11 @@
 Answer: YES</t>
         </is>
       </c>
+      <c r="D111" s="3" t="inlineStr"/>
+      <c r="E111" s="3" t="inlineStr"/>
+      <c r="F111" s="3" t="inlineStr"/>
       <c r="G111" s="3" t="inlineStr"/>
       <c r="H111" s="3" t="inlineStr"/>
-      <c r="I111" s="3" t="inlineStr"/>
-      <c r="J111" s="3" t="inlineStr"/>
-      <c r="K111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -20410,21 +19198,6 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-703']</t>
-        </is>
-      </c>
-      <c r="E112" s="2" t="inlineStr">
-        <is>
-          <t>TensorFlow is an open source platform for machine learning. Prior to versions 2.9.0, 2.8.1, 2.7.2, and 2.6.4, the implementation of `tf.raw_ops.LoadAndRemapMatrix does not fully validate the input arguments. This results in a `CHECK`-failure which can be used to trigger a denial of service attack. The code assumes `initializing_values` is a vector but there is no validation for this before accessing its value. Versions 2.9.0, 2.8.1, 2.7.2, and 2.6.4 contain a patch for this issue.</t>
-        </is>
-      </c>
-      <c r="F112" s="2" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 ### 1. **Input Validation**
 - The code checks the sizes of input tensors (`row_remapping`, `col_remapping`, `ckpt_path`, `old_tensor_name`, `initializing_values`) against expected values or constraints.
@@ -20453,19 +19226,19 @@
 - Consider additional security measures such as limiting the types of files that can be loaded or implementing file integrity checks.</t>
         </is>
       </c>
+      <c r="D112" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E112" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F112" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G112" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H112" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I112" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J112" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="K112" s="2" t="inlineStr">
+      <c r="H112" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -20665,21 +19438,6 @@
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-787']</t>
-        </is>
-      </c>
-      <c r="E113" s="3" t="inlineStr">
-        <is>
-          <t>Heap-based Buffer Overflow in GitHub repository vim/vim prior to 8.2.4436.</t>
-        </is>
-      </c>
-      <c r="F113" s="3" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 1. **Code Overview**:
 	* The provided code is a function `change_indent` written in C, likely part of the Vim text editor.
@@ -20711,11 +19469,11 @@
 - Consider adding more comprehensive error checking for function return values to ensure robustness against unexpected internal errors.</t>
         </is>
       </c>
+      <c r="D113" s="3" t="inlineStr"/>
+      <c r="E113" s="3" t="inlineStr"/>
+      <c r="F113" s="3" t="inlineStr"/>
       <c r="G113" s="3" t="inlineStr"/>
       <c r="H113" s="3" t="inlineStr"/>
-      <c r="I113" s="3" t="inlineStr"/>
-      <c r="J113" s="3" t="inlineStr"/>
-      <c r="K113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="n">
@@ -20786,21 +19544,6 @@
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D114" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-362']</t>
-        </is>
-      </c>
-      <c r="E114" s="3" t="inlineStr">
-        <is>
-          <t>World-writable permissions on the /tmp/tmate/sessions directory in tmate-ssh-server 2.3.0 allow a local attacker to compromise the integrity of session handling, or obtain the read-write session ID from a read-only session symlink in this directory.</t>
-        </is>
-      </c>
-      <c r="F114" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities:
 ### 1. **Input Handling via `getopt` and `xstrdup`**
 *   The code uses `getopt` to parse command-line options, which is a standard and secure approach.
@@ -20828,11 +19571,11 @@
 *   **Reason:** The use of `atoi` for converting user input to integers without error handling poses a potential vulnerability, as it can lead to unexpected behavior if non-integer inputs are provided for options expecting integer values. This could result in the application entering an unintended state, which might be exploitable in certain contexts. For example, incorrect port numbers could cause the SSH server to fail, leading to a denial of service. A more secure approach would be to use `strtol` or `strtoul`, which provide better error handling for such conversions.</t>
         </is>
       </c>
+      <c r="D114" s="3" t="inlineStr"/>
+      <c r="E114" s="3" t="inlineStr"/>
+      <c r="F114" s="3" t="inlineStr"/>
       <c r="G114" s="3" t="inlineStr"/>
       <c r="H114" s="3" t="inlineStr"/>
-      <c r="I114" s="3" t="inlineStr"/>
-      <c r="J114" s="3" t="inlineStr"/>
-      <c r="K114" s="3" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="n">
@@ -20886,21 +19629,6 @@
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D115" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-476']</t>
-        </is>
-      </c>
-      <c r="E115" s="3" t="inlineStr">
-        <is>
-          <t>An issue was discovered in the Linux kernel through 5.16-rc6. There is a lack of check after calling vzalloc() and lack of free after allocation in drivers/media/test-drivers/vidtv/vidtv_s302m.c.</t>
-        </is>
-      </c>
-      <c r="F115" s="3" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Unchecked Memory Allocations:**
@@ -20913,11 +19641,11 @@
 **Conclusion:** The code contains multiple vulnerabilities due to unchecked memory allocations and unsafe handling of input parameters. These issues can lead to NULL pointer dereferences, memory corruption, or denial-of-service conditions, making the code vulnerable.</t>
         </is>
       </c>
+      <c r="D115" s="3" t="inlineStr"/>
+      <c r="E115" s="3" t="inlineStr"/>
+      <c r="F115" s="3" t="inlineStr"/>
       <c r="G115" s="3" t="inlineStr"/>
       <c r="H115" s="3" t="inlineStr"/>
-      <c r="I115" s="3" t="inlineStr"/>
-      <c r="J115" s="3" t="inlineStr"/>
-      <c r="K115" s="3" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -21014,13 +19742,6 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D116" s="2" t="inlineStr"/>
-      <c r="E116" s="2" t="inlineStr"/>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step from a security and static program analysis perspective, focusing on potential vulnerabilities.
 **Code Overview**
 The code is part of a custom TensorFlow operation (`AssignOp`) that assigns the value of one tensor (`rhs`, right-hand side) to another (`lhs`, left-hand side). It handles tensor initialization, shape validation, memory allocation, and data copying, considering performance optimizations.
@@ -21049,19 +19770,19 @@
 The provided code snippet appears to be securely written, following best practices for input validation, memory management, concurrency control, and error handling within the context of TensorFlow custom operations. Without additional context or implementation details of surrounding code (e.g., the `Copy` function), no vulnerabilities are detected within this snippet.</t>
         </is>
       </c>
+      <c r="D116" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E116" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F116" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G116" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H116" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I116" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J116" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="K116" s="2" t="inlineStr">
+      <c r="H116" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -21236,13 +19957,6 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D117" s="2" t="inlineStr"/>
-      <c r="E117" s="2" t="inlineStr"/>
-      <c r="F117" s="2" t="inlineStr">
-        <is>
           <t>**Step-by-Step Analysis**
 1. **Code Overview**:
 	* The provided code is a part of the GnuTLS library, specifically the `_gnutls_server_select_suite` function.
@@ -21264,19 +19978,19 @@
 **Note**: This analysis is based on the provided code snippet. In a real-world scenario, understanding the entire codebase and the context in which this function is called would be crucial for a comprehensive security assessment.</t>
         </is>
       </c>
+      <c r="D117" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E117" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F117" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G117" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H117" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I117" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J117" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K117" s="2" t="inlineStr">
+      <c r="H117" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -21351,21 +20065,6 @@
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
-        <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D118" s="3" t="inlineStr">
-        <is>
-          <t>['CWE-703']</t>
-        </is>
-      </c>
-      <c r="E118" s="3" t="inlineStr">
-        <is>
-          <t>NULL Pointer Dereference in GitHub repository mruby/mruby prior to 3.2.</t>
-        </is>
-      </c>
-      <c r="F118" s="3" t="inlineStr">
         <is>
           <t>### Analysis of the Provided Code
 The function `fiber_switch` is part of a fiber implementation in a language like MRuby, responsible for switching between lightweight threads (fibers). It handles context switching, argument passing, and error checking based on the current state of the fiber.
@@ -21406,11 +20105,11 @@
 **(2) NO: No vulnerability.**</t>
         </is>
       </c>
+      <c r="D118" s="3" t="inlineStr"/>
+      <c r="E118" s="3" t="inlineStr"/>
+      <c r="F118" s="3" t="inlineStr"/>
       <c r="G118" s="3" t="inlineStr"/>
       <c r="H118" s="3" t="inlineStr"/>
-      <c r="I118" s="3" t="inlineStr"/>
-      <c r="J118" s="3" t="inlineStr"/>
-      <c r="K118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -21511,21 +20210,6 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-369']</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
-          <t>TensorFlow is an end-to-end open source platform for machine learning. In affected versions an attacker can craft a TFLite model that would trigger a null pointer dereference, which would result in a crash and denial of service. The [implementation](https://github.com/tensorflow/tensorflow/blob/149562d49faa709ea80df1d99fc41d005b81082a/tensorflow/lite/kernels/internal/optimized/optimized_ops.h#L268-L285) unconditionally dereferences a pointer. We have patched the issue in GitHub commit 15691e456c7dc9bd6be203b09765b063bf4a380c. The fix will be included in TensorFlow 2.6.0. We will also cherrypick this commit on TensorFlow 2.5.1, TensorFlow 2.4.3, and TensorFlow 2.3.4, as these are also affected and still in supported range.</t>
-        </is>
-      </c>
-      <c r="F119" s="2" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step from a security perspective, focusing on common vulnerabilities that can be detected through static program analysis:
 ### 1. **Input Validation**
 - **Observation**: The function takes multiple parameters including pointers to data (`unswitched_input1_data`, `unswitched_input2_data`, `output_data`) and their respective shapes. However, there's no explicit check for `NULL` pointers or validation of the shape dimensions against potential out-of-bounds accesses.
@@ -21549,19 +20233,19 @@
 4. **Use Secure Coding Practices**: Apply secure coding standards and guidelines (e.g., CERT C/C++ coding standards) to the entire codebase.</t>
         </is>
       </c>
+      <c r="D119" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E119" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F119" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="G119" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H119" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I119" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J119" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K119" s="2" t="inlineStr">
+      <c r="H119" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -21632,21 +20316,6 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>vulnerable</t>
-        </is>
-      </c>
-      <c r="D120" s="2" t="inlineStr">
-        <is>
-          <t>['CWE-125']</t>
-        </is>
-      </c>
-      <c r="E120" s="2" t="inlineStr">
-        <is>
-          <t>Tensorflow is an Open Source Machine Learning Framework. TensorFlow's type inference can cause a heap out of bounds read as the bounds checking is done in a `DCHECK` (which is a no-op during production). An attacker can control the `input_idx` variable such that `ix` would be larger than the number of values in `node_t.args`. The fix will be included in TensorFlow 2.8.0. This is the only affected version.</t>
-        </is>
-      </c>
-      <c r="F120" s="2" t="inlineStr">
-        <is>
           <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Input Validation and Edge Handling:**
@@ -21662,19 +20331,19 @@
 **Conclusion:** The absence of a release-mode bounds check for `args(ix)` access constitutes a vulnerability, making the answer **YES**.</t>
         </is>
       </c>
+      <c r="D120" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E120" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F120" s="2" t="n">
+        <v>4</v>
+      </c>
       <c r="G120" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="H120" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I120" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J120" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="K120" s="2" t="inlineStr">
+      <c r="H120" s="2" t="inlineStr">
         <is>
           <t>prior (already rated)</t>
         </is>
@@ -21772,13 +20441,6 @@
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>safe</t>
-        </is>
-      </c>
-      <c r="D121" s="3" t="inlineStr"/>
-      <c r="E121" s="3" t="inlineStr"/>
-      <c r="F121" s="3" t="inlineStr">
-        <is>
           <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
 **Function Overview**
 --------------------
@@ -21810,11 +20472,11 @@
 3. **Review `gf_fgets` and `gf_utf8_wcstombs`**: Ensure these functions adhere to secure coding practices, especially regarding buffer sizes and bounds checking.</t>
         </is>
       </c>
+      <c r="D121" s="3" t="inlineStr"/>
+      <c r="E121" s="3" t="inlineStr"/>
+      <c r="F121" s="3" t="inlineStr"/>
       <c r="G121" s="3" t="inlineStr"/>
       <c r="H121" s="3" t="inlineStr"/>
-      <c r="I121" s="3" t="inlineStr"/>
-      <c r="J121" s="3" t="inlineStr"/>
-      <c r="K121" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(rq3): replace broken FN snippet 215921 -> 213515 in the paired-120 set
idx=215921 thinking failed 3x (timeout + 2 empty completions) — no obtainable
thinking response, so its paired think-vs-instruct row (sample 9) could not be
rated. Replaced with a fresh valid FN snippet (idx=213515, gt=1, both modes pred=0,
CWE-787) in samples 9 (thinking) + 18 (instruct); frame now has 15 FN snippets and
zero skip/no-response responses. Repo rater sheets synced; minimal redistribution
patch fpfn_paired120_replacement_s9_s18.xlsx holds just those 2 rows so raters
update in place without losing in-progress work.
</commit_message>
<xml_diff>
--- a/results/rq3_baseline/fpfn_paired120_rater_HS.xlsx
+++ b/results/rq3_baseline/fpfn_paired120_rater_HS.xlsx
@@ -1236,85 +1236,252 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>bmexec_trans (kwset_t kwset, char const *text, size_t size)
+          <t>spell_suggest(int count)
 {
-  unsigned char const *d1;
-  char const *ep, *sp, *tp;
-  int d;
-  int len = kwset-&gt;mind;
-  char const *trans = kwset-&gt;trans;
-  if (len == 0)
-    return 0;
-  if (len &gt; size)
-    return -1;
-  if (len == 1)
+    char_u	*line;
+    pos_T	prev_cursor = curwin-&gt;w_cursor;
+    char_u	wcopy[MAXWLEN + 2];
+    char_u	*p;
+    int		i;
+    int		c;
+    suginfo_T	sug;
+    suggest_T	*stp;
+    int		mouse_used;
+    int		need_cap;
+    int		limit;
+    int		selected = count;
+    int		badlen = 0;
+    int		msg_scroll_save = msg_scroll;
+    int		wo_spell_save = curwin-&gt;w_p_spell;
+    if (!curwin-&gt;w_p_spell)
     {
-      tp = memchr_kwset (text, size, kwset);
-      return tp ? tp - text : -1;
-    }
-  d1 = kwset-&gt;delta;
-  sp = kwset-&gt;target + len;
-  tp = text + len;
-  char gc1 = kwset-&gt;gc1;
-  char gc2 = kwset-&gt;gc2;
-  /* Significance of 12: 1 (initial offset) + 10 (skip loop) + 1 (md2). */
-  if (size &gt; 12 * len)
-    /* 11 is not a bug, the initial offset happens only once. */
-    for (ep = text + size - 11 * len; tp &lt;= ep; )
-      {
-        char const *tp0 = tp;
-        d = d1[U(tp[-1])], tp += d;
-        d = d1[U(tp[-1])], tp += d;
-        if (d != 0)
-          {
-            d = d1[U(tp[-1])], tp += d;
-            d = d1[U(tp[-1])], tp += d;
-            d = d1[U(tp[-1])], tp += d;
-            if (d != 0)
-              {
-                d = d1[U(tp[-1])], tp += d;
-                d = d1[U(tp[-1])], tp += d;
-                d = d1[U(tp[-1])], tp += d;
-                if (d != 0)
-                  {
-                    d = d1[U(tp[-1])], tp += d;
-                    d = d1[U(tp[-1])], tp += d;
-                    /* As a heuristic, prefer memchr to seeking by
-                       delta1 when the latter doesn't advance much.  */
-                    int advance_heuristic = 16 * sizeof (long);
-                    if (advance_heuristic &lt;= tp - tp0)
-                      goto big_advance;
-                    tp--;
-                    tp = memchr_kwset (tp, text + size - tp, kwset);
-                    if (! tp)
-                      return -1;
-                    tp++;
-                  }
-              }
-          }
-        if (bm_delta2_search (&amp;tp, ep, sp, len, trans, gc1, gc2, d1, kwset))
-          return tp - text;
-      big_advance:;
-      }
-  /* Now we have only a few characters left to search.  We
-     carefully avoid ever producing an out-of-bounds pointer. */
-  ep = text + size;
-  d = d1[U(tp[-1])];
-  while (d &lt;= ep - tp)
+	did_set_spelllang(curwin);
+	curwin-&gt;w_p_spell = TRUE;
+    }
+    if (*curwin-&gt;w_s-&gt;b_p_spl == NUL)
     {
-      d = d1[U((tp += d)[-1])];
-      if (d != 0)
-        continue;
-      if (bm_delta2_search (&amp;tp, ep, sp, len, trans, gc1, gc2, NULL, kwset))
-        return tp - text;
-    }
-  return -1;
+	emsg(_(e_spell_checking_is_not_possible));
+	return;
+    }
+    if (VIsual_active)
+    {
+	// Use the Visually selected text as the bad word.  But reject
+	// a multi-line selection.
+	if (curwin-&gt;w_cursor.lnum != VIsual.lnum)
+	{
+	    vim_beep(BO_SPELL);
+	    return;
+	}
+	badlen = (int)curwin-&gt;w_cursor.col - (int)VIsual.col;
+	if (badlen &lt; 0)
+	    badlen = -badlen;
+	else
+	    curwin-&gt;w_cursor.col = VIsual.col;
+	++badlen;
+	end_visual_mode();
+    }
+    // Find the start of the badly spelled word.
+    else if (spell_move_to(curwin, FORWARD, TRUE, TRUE, NULL) == 0
+	    || curwin-&gt;w_cursor.col &gt; prev_cursor.col)
+    {
+	// No bad word or it starts after the cursor: use the word under the
+	// cursor.
+	curwin-&gt;w_cursor = prev_cursor;
+	line = ml_get_curline();
+	p = line + curwin-&gt;w_cursor.col;
+	// Backup to before start of word.
+	while (p &gt; line &amp;&amp; spell_iswordp_nmw(p, curwin))
+	    MB_PTR_BACK(line, p);
+	// Forward to start of word.
+	while (*p != NUL &amp;&amp; !spell_iswordp_nmw(p, curwin))
+	    MB_PTR_ADV(p);
+	if (!spell_iswordp_nmw(p, curwin))		// No word found.
+	{
+	    beep_flush();
+	    return;
+	}
+	curwin-&gt;w_cursor.col = (colnr_T)(p - line);
+    }
+    // Get the word and its length.
+    // Figure out if the word should be capitalised.
+    need_cap = check_need_cap(curwin-&gt;w_cursor.lnum, curwin-&gt;w_cursor.col);
+    // Make a copy of current line since autocommands may free the line.
+    line = vim_strsave(ml_get_curline());
+    if (line == NULL)
+	goto skip;
+    // Get the list of suggestions.  Limit to 'lines' - 2 or the number in
+    // 'spellsuggest', whatever is smaller.
+    if (sps_limit &gt; (int)Rows - 2)
+	limit = (int)Rows - 2;
+    else
+	limit = sps_limit;
+    spell_find_suggest(line + curwin-&gt;w_cursor.col, badlen, &amp;sug, limit,
+							TRUE, need_cap, TRUE);
+    if (sug.su_ga.ga_len == 0)
+	msg(_("Sorry, no suggestions"));
+    else if (count &gt; 0)
+    {
+	if (count &gt; sug.su_ga.ga_len)
+	    smsg(_("Sorry, only %ld suggestions"), (long)sug.su_ga.ga_len);
+    }
+    else
+    {
+#ifdef FEAT_RIGHTLEFT
+	// When 'rightleft' is set the list is drawn right-left.
+	cmdmsg_rl = curwin-&gt;w_p_rl;
+	if (cmdmsg_rl)
+	    msg_col = Columns - 1;
+#endif
+	// List the suggestions.
+	msg_start();
+	msg_row = Rows - 1;	// for when 'cmdheight' &gt; 1
+	lines_left = Rows;	// avoid more prompt
+	vim_snprintf((char *)IObuff, IOSIZE, _("Change \"%.*s\" to:"),
+						sug.su_badlen, sug.su_badptr);
+#ifdef FEAT_RIGHTLEFT
+	if (cmdmsg_rl &amp;&amp; STRNCMP(IObuff, "Change", 6) == 0)
+	{
+	    // And now the rabbit from the high hat: Avoid showing the
+	    // untranslated message rightleft.
+	    vim_snprintf((char *)IObuff, IOSIZE, ":ot \"%.*s\" egnahC",
+						sug.su_badlen, sug.su_badptr);
+	}
+#endif
+	msg_puts((char *)IObuff);
+	msg_clr_eos();
+	msg_putchar('\n');
+	msg_scroll = TRUE;
+	for (i = 0; i &lt; sug.su_ga.ga_len; ++i)
+	{
+	    stp = &amp;SUG(sug.su_ga, i);
+	    // The suggested word may replace only part of the bad word, add
+	    // the not replaced part.
+	    vim_strncpy(wcopy, stp-&gt;st_word, MAXWLEN);
+	    if (sug.su_badlen &gt; stp-&gt;st_orglen)
+		vim_strncpy(wcopy + stp-&gt;st_wordlen,
+					       sug.su_badptr + stp-&gt;st_orglen,
+					      sug.su_badlen - stp-&gt;st_orglen);
+	    vim_snprintf((char *)IObuff, IOSIZE, "%2d", i + 1);
+#ifdef FEAT_RIGHTLEFT
+	    if (cmdmsg_rl)
+		rl_mirror(IObuff);
+#endif
+	    msg_puts((char *)IObuff);
+	    vim_snprintf((char *)IObuff, IOSIZE, " \"%s\"", wcopy);
+	    msg_puts((char *)IObuff);
+	    // The word may replace more than "su_badlen".
+	    if (sug.su_badlen &lt; stp-&gt;st_orglen)
+	    {
+		vim_snprintf((char *)IObuff, IOSIZE, _(" &lt; \"%.*s\""),
+					       stp-&gt;st_orglen, sug.su_badptr);
+		msg_puts((char *)IObuff);
+	    }
+	    if (p_verbose &gt; 0)
+	    {
+		// Add the score.
+		if (sps_flags &amp; (SPS_DOUBLE | SPS_BEST))
+		    vim_snprintf((char *)IObuff, IOSIZE, " (%s%d - %d)",
+			stp-&gt;st_salscore ? "s " : "",
+			stp-&gt;st_score, stp-&gt;st_altscore);
+		else
+		    vim_snprintf((char *)IObuff, IOSIZE, " (%d)",
+			    stp-&gt;st_score);
+#ifdef FEAT_RIGHTLEFT
+		if (cmdmsg_rl)
+		    // Mirror the numbers, but keep the leading space.
+		    rl_mirror(IObuff + 1);
+#endif
+		msg_advance(30);
+		msg_puts((char *)IObuff);
+	    }
+	    msg_putchar('\n');
+	}
+#ifdef FEAT_RIGHTLEFT
+	cmdmsg_rl = FALSE;
+	msg_col = 0;
+#endif
+	// Ask for choice.
+	selected = prompt_for_number(&amp;mouse_used);
+	if (mouse_used)
+	    selected -= lines_left;
+	lines_left = Rows;		// avoid more prompt
+	// don't delay for 'smd' in normal_cmd()
+	msg_scroll = msg_scroll_save;
+    }
+    if (selected &gt; 0 &amp;&amp; selected &lt;= sug.su_ga.ga_len &amp;&amp; u_save_cursor() == OK)
+    {
+	// Save the from and to text for :spellrepall.
+	VIM_CLEAR(repl_from);
+	VIM_CLEAR(repl_to);
+	stp = &amp;SUG(sug.su_ga, selected - 1);
+	if (sug.su_badlen &gt; stp-&gt;st_orglen)
+	{
+	    // Replacing less than "su_badlen", append the remainder to
+	    // repl_to.
+	    repl_from = vim_strnsave(sug.su_badptr, sug.su_badlen);
+	    vim_snprintf((char *)IObuff, IOSIZE, "%s%.*s", stp-&gt;st_word,
+		    sug.su_badlen - stp-&gt;st_orglen,
+					      sug.su_badptr + stp-&gt;st_orglen);
+	    repl_to = vim_strsave(IObuff);
+	}
+	else
+	{
+	    // Replacing su_badlen or more, use the whole word.
+	    repl_from = vim_strnsave(sug.su_badptr, stp-&gt;st_orglen);
+	    repl_to = vim_strsave(stp-&gt;st_word);
+	}
+	// Replace the word.
+	p = alloc(STRLEN(line) - stp-&gt;st_orglen + stp-&gt;st_wordlen + 1);
+	if (p != NULL)
+	{
+	    c = (int)(sug.su_badptr - line);
+	    mch_memmove(p, line, c);
+	    STRCPY(p + c, stp-&gt;st_word);
+	    STRCAT(p, sug.su_badptr + stp-&gt;st_orglen);
+	    // For redo we use a change-word command.
+	    ResetRedobuff();
+	    AppendToRedobuff((char_u *)"ciw");
+	    AppendToRedobuffLit(p + c,
+			    stp-&gt;st_wordlen + sug.su_badlen - stp-&gt;st_orglen);
+	    AppendCharToRedobuff(ESC);
+	    // "p" may be freed here
+	    ml_replace(curwin-&gt;w_cursor.lnum, p, FALSE);
+	    curwin-&gt;w_cursor.col = c;
+	    changed_bytes(curwin-&gt;w_cursor.lnum, c);
+	}
+    }
+    else
+	curwin-&gt;w_cursor = prev_cursor;
+    spell_find_cleanup(&amp;sug);
+skip:
+    vim_free(line);
+    curwin-&gt;w_p_spell = wo_spell_save;
 }</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>SKIPPED: timeout</t>
+          <t>**Step-by-Step Analysis**
+### 1. **Code Overview**
+The provided code is a function `spell_suggest` written in C, which appears to be part of a text editor (likely Vim, given the context and function names). The function is responsible for suggesting spell corrections for a misspelled word in the editor.
+### 2. **Input Handling**
+- **Direct Inputs**: The function indirectly receives input through the editor's state (e.g., `curwin-&gt;w_cursor`, `VIsual`, `curwin-&gt;w_p_spell`, etc.). Direct user input is handled through the editor's interface, not directly within this function.
+- **Input Validation**: The code checks for various conditions (e.g., if spell checking is enabled, if a visual selection is valid, etc.), but these are more related to functionality than security validation.
+### 3. **Potential Vulnerability Areas**
+- **Buffer Overflows**:
+	+ `vim_strncpy(wcopy, stp-&gt;st_word, MAXWLEN);` and similar uses of `vim_strncpy` are relatively safe due to the specified buffer size.
+	+ `vim_snprintf((char *)IObuff, IOSIZE, ...)` also seems safe due to the buffer size specification.
+- **Memory Management**:
+	+ `line = vim_strsave(ml_get_curline());` and `p = alloc(...)` are checked for `NULL`, indicating an attempt to handle allocation failures.
+	+ `vim_free(line);` is called at the end to free allocated memory, reducing the risk of memory leaks.
+- **User Input Handling in Suggestion List**:
+	+ The function `prompt_for_number(&amp;mouse_used);` is used to get user input for selecting a suggestion. However, the validation of this input is minimal: `if (selected &gt; 0 &amp;&amp; selected &lt;= sug.su_ga.ga_len &amp;&amp; u_save_cursor() == OK)`. While it checks the range, it assumes `prompt_for_number` will always return a numeric value, which might not be the case if the function is manipulated or if there's an underlying issue with how it handles non-numeric input.
+### 4. **Vulnerability Detection**
+Based on the analysis, the primary concern is the assumption that `prompt_for_number` will always return a valid numeric input within the expected range. If this function can be manipulated to return non-numeric values or values outside the expected range, it could potentially lead to unexpected behavior. However, without the implementation details of `prompt_for_number`, it's challenging to definitively state this as a vulnerability.
+**Result:**
+Given the information and focusing strictly on the provided code snippet:
+**(2) NO: No vulnerability.**
+**Rationale**: The code snippet does not explicitly contain common vulnerabilities such as buffer overflows, unchecked input, or unsafe memory practices that directly lead to security issues. The primary concern (input validation for `prompt_for_number`) is speculative without more context on its implementation.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr"/>
@@ -3824,105 +3991,250 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>bmexec_trans (kwset_t kwset, char const *text, size_t size)
+          <t>spell_suggest(int count)
 {
-  unsigned char const *d1;
-  char const *ep, *sp, *tp;
-  int d;
-  int len = kwset-&gt;mind;
-  char const *trans = kwset-&gt;trans;
-  if (len == 0)
-    return 0;
-  if (len &gt; size)
-    return -1;
-  if (len == 1)
+    char_u	*line;
+    pos_T	prev_cursor = curwin-&gt;w_cursor;
+    char_u	wcopy[MAXWLEN + 2];
+    char_u	*p;
+    int		i;
+    int		c;
+    suginfo_T	sug;
+    suggest_T	*stp;
+    int		mouse_used;
+    int		need_cap;
+    int		limit;
+    int		selected = count;
+    int		badlen = 0;
+    int		msg_scroll_save = msg_scroll;
+    int		wo_spell_save = curwin-&gt;w_p_spell;
+    if (!curwin-&gt;w_p_spell)
     {
-      tp = memchr_kwset (text, size, kwset);
-      return tp ? tp - text : -1;
-    }
-  d1 = kwset-&gt;delta;
-  sp = kwset-&gt;target + len;
-  tp = text + len;
-  char gc1 = kwset-&gt;gc1;
-  char gc2 = kwset-&gt;gc2;
-  /* Significance of 12: 1 (initial offset) + 10 (skip loop) + 1 (md2). */
-  if (size &gt; 12 * len)
-    /* 11 is not a bug, the initial offset happens only once. */
-    for (ep = text + size - 11 * len; tp &lt;= ep; )
-      {
-        char const *tp0 = tp;
-        d = d1[U(tp[-1])], tp += d;
-        d = d1[U(tp[-1])], tp += d;
-        if (d != 0)
-          {
-            d = d1[U(tp[-1])], tp += d;
-            d = d1[U(tp[-1])], tp += d;
-            d = d1[U(tp[-1])], tp += d;
-            if (d != 0)
-              {
-                d = d1[U(tp[-1])], tp += d;
-                d = d1[U(tp[-1])], tp += d;
-                d = d1[U(tp[-1])], tp += d;
-                if (d != 0)
-                  {
-                    d = d1[U(tp[-1])], tp += d;
-                    d = d1[U(tp[-1])], tp += d;
-                    /* As a heuristic, prefer memchr to seeking by
-                       delta1 when the latter doesn't advance much.  */
-                    int advance_heuristic = 16 * sizeof (long);
-                    if (advance_heuristic &lt;= tp - tp0)
-                      goto big_advance;
-                    tp--;
-                    tp = memchr_kwset (tp, text + size - tp, kwset);
-                    if (! tp)
-                      return -1;
-                    tp++;
-                  }
-              }
-          }
-        if (bm_delta2_search (&amp;tp, ep, sp, len, trans, gc1, gc2, d1, kwset))
-          return tp - text;
-      big_advance:;
-      }
-  /* Now we have only a few characters left to search.  We
-     carefully avoid ever producing an out-of-bounds pointer. */
-  ep = text + size;
-  d = d1[U(tp[-1])];
-  while (d &lt;= ep - tp)
+	did_set_spelllang(curwin);
+	curwin-&gt;w_p_spell = TRUE;
+    }
+    if (*curwin-&gt;w_s-&gt;b_p_spl == NUL)
     {
-      d = d1[U((tp += d)[-1])];
-      if (d != 0)
-        continue;
-      if (bm_delta2_search (&amp;tp, ep, sp, len, trans, gc1, gc2, NULL, kwset))
-        return tp - text;
-    }
-  return -1;
+	emsg(_(e_spell_checking_is_not_possible));
+	return;
+    }
+    if (VIsual_active)
+    {
+	// Use the Visually selected text as the bad word.  But reject
+	// a multi-line selection.
+	if (curwin-&gt;w_cursor.lnum != VIsual.lnum)
+	{
+	    vim_beep(BO_SPELL);
+	    return;
+	}
+	badlen = (int)curwin-&gt;w_cursor.col - (int)VIsual.col;
+	if (badlen &lt; 0)
+	    badlen = -badlen;
+	else
+	    curwin-&gt;w_cursor.col = VIsual.col;
+	++badlen;
+	end_visual_mode();
+    }
+    // Find the start of the badly spelled word.
+    else if (spell_move_to(curwin, FORWARD, TRUE, TRUE, NULL) == 0
+	    || curwin-&gt;w_cursor.col &gt; prev_cursor.col)
+    {
+	// No bad word or it starts after the cursor: use the word under the
+	// cursor.
+	curwin-&gt;w_cursor = prev_cursor;
+	line = ml_get_curline();
+	p = line + curwin-&gt;w_cursor.col;
+	// Backup to before start of word.
+	while (p &gt; line &amp;&amp; spell_iswordp_nmw(p, curwin))
+	    MB_PTR_BACK(line, p);
+	// Forward to start of word.
+	while (*p != NUL &amp;&amp; !spell_iswordp_nmw(p, curwin))
+	    MB_PTR_ADV(p);
+	if (!spell_iswordp_nmw(p, curwin))		// No word found.
+	{
+	    beep_flush();
+	    return;
+	}
+	curwin-&gt;w_cursor.col = (colnr_T)(p - line);
+    }
+    // Get the word and its length.
+    // Figure out if the word should be capitalised.
+    need_cap = check_need_cap(curwin-&gt;w_cursor.lnum, curwin-&gt;w_cursor.col);
+    // Make a copy of current line since autocommands may free the line.
+    line = vim_strsave(ml_get_curline());
+    if (line == NULL)
+	goto skip;
+    // Get the list of suggestions.  Limit to 'lines' - 2 or the number in
+    // 'spellsuggest', whatever is smaller.
+    if (sps_limit &gt; (int)Rows - 2)
+	limit = (int)Rows - 2;
+    else
+	limit = sps_limit;
+    spell_find_suggest(line + curwin-&gt;w_cursor.col, badlen, &amp;sug, limit,
+							TRUE, need_cap, TRUE);
+    if (sug.su_ga.ga_len == 0)
+	msg(_("Sorry, no suggestions"));
+    else if (count &gt; 0)
+    {
+	if (count &gt; sug.su_ga.ga_len)
+	    smsg(_("Sorry, only %ld suggestions"), (long)sug.su_ga.ga_len);
+    }
+    else
+    {
+#ifdef FEAT_RIGHTLEFT
+	// When 'rightleft' is set the list is drawn right-left.
+	cmdmsg_rl = curwin-&gt;w_p_rl;
+	if (cmdmsg_rl)
+	    msg_col = Columns - 1;
+#endif
+	// List the suggestions.
+	msg_start();
+	msg_row = Rows - 1;	// for when 'cmdheight' &gt; 1
+	lines_left = Rows;	// avoid more prompt
+	vim_snprintf((char *)IObuff, IOSIZE, _("Change \"%.*s\" to:"),
+						sug.su_badlen, sug.su_badptr);
+#ifdef FEAT_RIGHTLEFT
+	if (cmdmsg_rl &amp;&amp; STRNCMP(IObuff, "Change", 6) == 0)
+	{
+	    // And now the rabbit from the high hat: Avoid showing the
+	    // untranslated message rightleft.
+	    vim_snprintf((char *)IObuff, IOSIZE, ":ot \"%.*s\" egnahC",
+						sug.su_badlen, sug.su_badptr);
+	}
+#endif
+	msg_puts((char *)IObuff);
+	msg_clr_eos();
+	msg_putchar('\n');
+	msg_scroll = TRUE;
+	for (i = 0; i &lt; sug.su_ga.ga_len; ++i)
+	{
+	    stp = &amp;SUG(sug.su_ga, i);
+	    // The suggested word may replace only part of the bad word, add
+	    // the not replaced part.
+	    vim_strncpy(wcopy, stp-&gt;st_word, MAXWLEN);
+	    if (sug.su_badlen &gt; stp-&gt;st_orglen)
+		vim_strncpy(wcopy + stp-&gt;st_wordlen,
+					       sug.su_badptr + stp-&gt;st_orglen,
+					      sug.su_badlen - stp-&gt;st_orglen);
+	    vim_snprintf((char *)IObuff, IOSIZE, "%2d", i + 1);
+#ifdef FEAT_RIGHTLEFT
+	    if (cmdmsg_rl)
+		rl_mirror(IObuff);
+#endif
+	    msg_puts((char *)IObuff);
+	    vim_snprintf((char *)IObuff, IOSIZE, " \"%s\"", wcopy);
+	    msg_puts((char *)IObuff);
+	    // The word may replace more than "su_badlen".
+	    if (sug.su_badlen &lt; stp-&gt;st_orglen)
+	    {
+		vim_snprintf((char *)IObuff, IOSIZE, _(" &lt; \"%.*s\""),
+					       stp-&gt;st_orglen, sug.su_badptr);
+		msg_puts((char *)IObuff);
+	    }
+	    if (p_verbose &gt; 0)
+	    {
+		// Add the score.
+		if (sps_flags &amp; (SPS_DOUBLE | SPS_BEST))
+		    vim_snprintf((char *)IObuff, IOSIZE, " (%s%d - %d)",
+			stp-&gt;st_salscore ? "s " : "",
+			stp-&gt;st_score, stp-&gt;st_altscore);
+		else
+		    vim_snprintf((char *)IObuff, IOSIZE, " (%d)",
+			    stp-&gt;st_score);
+#ifdef FEAT_RIGHTLEFT
+		if (cmdmsg_rl)
+		    // Mirror the numbers, but keep the leading space.
+		    rl_mirror(IObuff + 1);
+#endif
+		msg_advance(30);
+		msg_puts((char *)IObuff);
+	    }
+	    msg_putchar('\n');
+	}
+#ifdef FEAT_RIGHTLEFT
+	cmdmsg_rl = FALSE;
+	msg_col = 0;
+#endif
+	// Ask for choice.
+	selected = prompt_for_number(&amp;mouse_used);
+	if (mouse_used)
+	    selected -= lines_left;
+	lines_left = Rows;		// avoid more prompt
+	// don't delay for 'smd' in normal_cmd()
+	msg_scroll = msg_scroll_save;
+    }
+    if (selected &gt; 0 &amp;&amp; selected &lt;= sug.su_ga.ga_len &amp;&amp; u_save_cursor() == OK)
+    {
+	// Save the from and to text for :spellrepall.
+	VIM_CLEAR(repl_from);
+	VIM_CLEAR(repl_to);
+	stp = &amp;SUG(sug.su_ga, selected - 1);
+	if (sug.su_badlen &gt; stp-&gt;st_orglen)
+	{
+	    // Replacing less than "su_badlen", append the remainder to
+	    // repl_to.
+	    repl_from = vim_strnsave(sug.su_badptr, sug.su_badlen);
+	    vim_snprintf((char *)IObuff, IOSIZE, "%s%.*s", stp-&gt;st_word,
+		    sug.su_badlen - stp-&gt;st_orglen,
+					      sug.su_badptr + stp-&gt;st_orglen);
+	    repl_to = vim_strsave(IObuff);
+	}
+	else
+	{
+	    // Replacing su_badlen or more, use the whole word.
+	    repl_from = vim_strnsave(sug.su_badptr, stp-&gt;st_orglen);
+	    repl_to = vim_strsave(stp-&gt;st_word);
+	}
+	// Replace the word.
+	p = alloc(STRLEN(line) - stp-&gt;st_orglen + stp-&gt;st_wordlen + 1);
+	if (p != NULL)
+	{
+	    c = (int)(sug.su_badptr - line);
+	    mch_memmove(p, line, c);
+	    STRCPY(p + c, stp-&gt;st_word);
+	    STRCAT(p, sug.su_badptr + stp-&gt;st_orglen);
+	    // For redo we use a change-word command.
+	    ResetRedobuff();
+	    AppendToRedobuff((char_u *)"ciw");
+	    AppendToRedobuffLit(p + c,
+			    stp-&gt;st_wordlen + sug.su_badlen - stp-&gt;st_orglen);
+	    AppendCharToRedobuff(ESC);
+	    // "p" may be freed here
+	    ml_replace(curwin-&gt;w_cursor.lnum, p, FALSE);
+	    curwin-&gt;w_cursor.col = c;
+	    changed_bytes(curwin-&gt;w_cursor.lnum, c);
+	}
+    }
+    else
+	curwin-&gt;w_cursor = prev_cursor;
+    spell_find_cleanup(&amp;sug);
+skip:
+    vim_free(line);
+    curwin-&gt;w_p_spell = wo_spell_save;
 }</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Let's analyze the provided code step-by-step for potential vulnerabilities.
-**Code Overview**
-The function `bmexec_trans` appears to be part of a string searching algorithm, likely an optimized variant of the Boyer-Moore algorithm, given the use of delta (difference) tables and heuristics for skipping characters. It searches for a pattern (defined by `kwset`) within a text buffer (`text` of size `size`).
-**Step-by-Step Analysis for Vulnerabilities**
-1. **Input Validation**:
-   - The function checks if `len` (derived from `kwset-&gt;mind`) is 0, returning immediately.
-   - It verifies if `len` exceeds `size`, returning -1 in such cases.
-   - **Partial Input Validation**: While it checks for `len == 0` and `len &gt; size`, it assumes `kwset`, `text`, and `size` are valid without explicit null or range checks for all inputs.
-2. **Memory Access**:
-   - The use of `memchr_kwset` (a custom function, presumably similar to `memchr` but with additional `kwset` logic) and manual pointer arithmetic (`tp[-1]`, `tp += d`, etc.) could potentially lead to out-of-bounds access if not carefully managed.
-   - **Potential Issue**: In the line `d = d1[U(tp[-1])]`, if `tp` is at the start of `text` (i.e., `tp == text`), `tp[-1]` would access memory out-of-bounds. However, the context suggests `tp` is advanced from `text + len`, making this scenario unlikely under normal operation but possible if `len` is 0 (already checked) or negative (not checked).
-3. **Pointer Arithmetic and Loops**:
-   - The function engages in complex pointer arithmetic and looping constructs, which can be prone to off-by-one errors or infinite loops if not perfectly balanced.
-   - **Observation**: The loops and pointer advancements appear to be carefully balanced with conditions to prevent infinite loops (e.g., `tp &lt;= ep`), but the complexity increases the risk of logical errors.
-4. **Use of Heuristics and Assumptions**:
-   - The heuristic for `advance_heuristic` and the decision to use `memchr_kwset` under certain conditions rely on assumptions about the data and system (e.g., `sizeof(long)`).
-   - **Potential Issue**: These assumptions might not hold in all environments or with all inputs, potentially leading to suboptimal performance or, in extreme cases, vulnerabilities if the heuristics lead to out-of-bounds access or infinite loops.
-**Conclusion**
-Given the analysis, while the code is complex and has some assumptions that could lead to performance issues or rare edge cases, **no clear, direct vulnerability (such as a buffer overflow, use-after-free, or format string vulnerability) is immediately apparent** from the provided snippet. The code seems to attempt careful handling of memory and bounds, albeit with some risk due to its complexity and reliance on certain assumptions.
+          <t>**Step-by-Step Analysis**
+### 1. **Code Overview**
+The provided code is a function `spell_suggest` written in C, which appears to be part of a text editor (likely Vim, given the context and function names). The function is responsible for suggesting spelling corrections for a misspelled word in the editor.
+### 2. **Input Handling**
+- **Direct Inputs**: The function indirectly receives input through the editor's current state (e.g., `curwin-&gt;w_cursor`, `curwin-&gt;w_p_spell`, etc.). Direct user input is handled through the editor's interface, not directly within this function.
+- **Input Validation**: The code checks for various conditions (e.g., if spelling is enabled, if a word is selected, etc.), but these are more about the editor's state than validating user input for security.
+### 3. **Potential Vulnerability Areas**
+- **Buffer Overflows**: The use of `vim_strncpy` and `vim_snprintf` is generally safer than their standard C counterparts, as they prevent buffer overflows by limiting the number of characters copied or printed.
+- **Memory Management**: The code uses `vim_strsave`, `alloc`, and `vim_free` for memory management, which are likely part of the editor's safe memory handling functions.
+- **User Input Handling**: Since the function doesn't directly handle user input (it relies on the editor's state), the risk of common vulnerabilities like SQL Injection or Cross-Site Scripting (XSS) is non-existent here.
+### 4. **Specific Vulnerability Check**
+- **Line Highlighting for Potential Issues**:
+  - `vim_strncpy(wcopy, stp-&gt;st_word, MAXWLEN);` **(Safe)**: Limits copy to `MAXWLEN`.
+  - `vim_snprintf((char *)IObuff, IOSIZE, ...)` **(Safe)**: Uses a size-limited sprintf variant.
+  - `alloc(STRLEN(line) - stp-&gt;st_orglen + stp-&gt;st_wordlen + 1)` **(Potential Risk)**: While it allocates memory based on calculated size, ensuring the correctness of `STRLEN(line)`, `stp-&gt;st_orglen`, and `stp-&gt;st_wordlen` is crucial. Incorrect calculations could lead to memory issues, but there's no direct indication of such errors in the provided snippet.
+### 5. **Conclusion**
+Based on the provided code snippet and analysis, there is **no clear vulnerability** detected within the `spell_suggest` function as it stands. The code appears to utilize safe functions for string and memory operations, and it does not directly handle user input in a manner that would introduce common security vulnerabilities.
 **Result: (2) NO: No vulnerability.**
-**Caveat**: This analysis is based on the provided code snippet and assumes the surrounding code and environment (e.g., how `kwset` is initialized, the implementation of `memchr_kwset`, and the `bm_delta2_search` function) do not introduce vulnerabilities. A full codebase review would be necessary for absolute certainty.</t>
+**Note**: This analysis is limited to the provided code snippet. The overall security of the application depends on various factors, including how this function is called, the security of surrounding code, and the handling of user input at the application level.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr"/>

</xml_diff>